<commit_message>
yerden2: tasarımda kapsama doğrulaması; tefriş/taşma 0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RwXcqZmf9VPBpDgb8LPkn3
</commit_message>
<xml_diff>
--- a/proje/denemeler/yerden2/NB_YERDEN_ISITMA.xlsx
+++ b/proje/denemeler/yerden2/NB_YERDEN_ISITMA.xlsx
@@ -5060,7 +5060,7 @@
         </is>
       </c>
       <c r="D18" s="343" t="n">
-        <v>2858.4</v>
+        <v>2125.2</v>
       </c>
       <c r="E18" s="344" t="n">
         <v>17.5</v>
@@ -5070,7 +5070,7 @@
         <v/>
       </c>
       <c r="G18" s="340" t="n">
-        <v>81.67</v>
+        <v>60.72</v>
       </c>
       <c r="H18" s="340" t="n">
         <v>2</v>
@@ -5330,7 +5330,7 @@
         </is>
       </c>
       <c r="D24" s="343" t="n">
-        <v>1334.6</v>
+        <v>1006.6</v>
       </c>
       <c r="E24" s="344" t="n">
         <v>17.5</v>
@@ -5340,7 +5340,7 @@
         <v/>
       </c>
       <c r="G24" s="340" t="n">
-        <v>38.13</v>
+        <v>28.76</v>
       </c>
       <c r="H24" s="340" t="n">
         <v>1</v>
@@ -6701,7 +6701,7 @@
         </is>
       </c>
       <c r="D55" s="348" t="n">
-        <v>1594.6</v>
+        <v>1586.9</v>
       </c>
       <c r="E55" s="349" t="n">
         <v>17.5</v>
@@ -6711,7 +6711,7 @@
         <v/>
       </c>
       <c r="G55" s="345" t="n">
-        <v>45.56</v>
+        <v>45.34</v>
       </c>
       <c r="H55" s="345" t="n">
         <v>1</v>
@@ -6746,7 +6746,7 @@
         </is>
       </c>
       <c r="D56" s="348" t="n">
-        <v>2847.9</v>
+        <v>2443.7</v>
       </c>
       <c r="E56" s="349" t="n">
         <v>17.5</v>
@@ -6756,7 +6756,7 @@
         <v/>
       </c>
       <c r="G56" s="345" t="n">
-        <v>81.37</v>
+        <v>69.81999999999999</v>
       </c>
       <c r="H56" s="345" t="n">
         <v>2</v>
@@ -7061,7 +7061,7 @@
         </is>
       </c>
       <c r="D63" s="348" t="n">
-        <v>2652.3</v>
+        <v>1210.3</v>
       </c>
       <c r="E63" s="349" t="n">
         <v>17.5</v>
@@ -7071,7 +7071,7 @@
         <v/>
       </c>
       <c r="G63" s="345" t="n">
-        <v>75.78</v>
+        <v>34.58</v>
       </c>
       <c r="H63" s="345" t="n">
         <v>2</v>
@@ -13241,7 +13241,7 @@
       </c>
       <c r="E2" s="383" t="inlineStr">
         <is>
-          <t>TOPLAM ISI = 37157 W</t>
+          <t>TOPLAM ISI = 36095 W</t>
         </is>
       </c>
       <c r="F2" s="264" t="n"/>
@@ -13952,10 +13952,10 @@
         <v>7.87</v>
       </c>
       <c r="P12" s="397" t="n">
-        <v>6.98</v>
+        <v>6.92</v>
       </c>
       <c r="Q12" s="397" t="n">
-        <v>6.49</v>
+        <v>6.55</v>
       </c>
       <c r="R12" s="397" t="n">
         <v>8.73</v>
@@ -14040,10 +14040,10 @@
         <v>1694</v>
       </c>
       <c r="P13" s="398" t="n">
-        <v>1480.5</v>
+        <v>1091.3</v>
       </c>
       <c r="Q13" s="398" t="n">
-        <v>1377.9</v>
+        <v>1033.9</v>
       </c>
       <c r="R13" s="398" t="n">
         <v>1365.3</v>
@@ -14064,7 +14064,7 @@
         <v>385.7</v>
       </c>
       <c r="X13" s="398" t="n">
-        <v>1334.6</v>
+        <v>1006.6</v>
       </c>
       <c r="Y13" s="398" t="n">
         <v>949.5</v>
@@ -16052,10 +16052,10 @@
         <v>9141</v>
       </c>
       <c r="P32" s="407" t="n">
-        <v>6311</v>
+        <v>2728</v>
       </c>
       <c r="Q32" s="407" t="n">
-        <v>5180</v>
+        <v>2351</v>
       </c>
       <c r="R32" s="407" t="n">
         <v>5051</v>
@@ -16076,7 +16076,7 @@
         <v>131</v>
       </c>
       <c r="X32" s="407" t="n">
-        <v>4745</v>
+        <v>2185</v>
       </c>
       <c r="Y32" s="407" t="n">
         <v>1861</v>
@@ -20704,7 +20704,7 @@
       </c>
       <c r="E2" s="383" t="inlineStr">
         <is>
-          <t>TOPLAM ISI = 36764 W</t>
+          <t>TOPLAM ISI = 34910 W</t>
         </is>
       </c>
       <c r="F2" s="264" t="n"/>
@@ -21500,10 +21500,10 @@
         <v>7.57</v>
       </c>
       <c r="G12" s="397" t="n">
-        <v>6.98</v>
+        <v>6.05</v>
       </c>
       <c r="H12" s="397" t="n">
-        <v>6.46</v>
+        <v>7.39</v>
       </c>
       <c r="I12" s="397" t="n">
         <v>8.73</v>
@@ -21527,10 +21527,10 @@
         <v>6.92</v>
       </c>
       <c r="P12" s="397" t="n">
-        <v>7.56</v>
+        <v>6.75</v>
       </c>
       <c r="Q12" s="397" t="n">
-        <v>6.46</v>
+        <v>7.27</v>
       </c>
       <c r="R12" s="397" t="n">
         <v>8.66</v>
@@ -21602,13 +21602,13 @@
       <c r="D13" s="261" t="n"/>
       <c r="E13" s="259" t="n"/>
       <c r="F13" s="398" t="n">
-        <v>1594.6</v>
+        <v>1586.9</v>
       </c>
       <c r="G13" s="398" t="n">
-        <v>1478</v>
+        <v>1100</v>
       </c>
       <c r="H13" s="398" t="n">
-        <v>1369.9</v>
+        <v>1343.7</v>
       </c>
       <c r="I13" s="398" t="n">
         <v>1361.2</v>
@@ -21632,10 +21632,10 @@
         <v>1189.3</v>
       </c>
       <c r="P13" s="398" t="n">
-        <v>1429.8</v>
+        <v>583.1</v>
       </c>
       <c r="Q13" s="398" t="n">
-        <v>1222.5</v>
+        <v>627.2</v>
       </c>
       <c r="R13" s="398" t="n">
         <v>1539</v>
@@ -23930,13 +23930,13 @@
       </c>
       <c r="E32" s="259" t="n"/>
       <c r="F32" s="407" t="n">
-        <v>7741</v>
+        <v>7639</v>
       </c>
       <c r="G32" s="407" t="n">
-        <v>6282</v>
+        <v>2788</v>
       </c>
       <c r="H32" s="407" t="n">
-        <v>5098</v>
+        <v>4834</v>
       </c>
       <c r="I32" s="407" t="n">
         <v>5009</v>
@@ -23960,10 +23960,10 @@
         <v>3456</v>
       </c>
       <c r="P32" s="407" t="n">
-        <v>5734</v>
+        <v>300</v>
       </c>
       <c r="Q32" s="407" t="n">
-        <v>3728</v>
+        <v>595</v>
       </c>
       <c r="R32" s="407" t="n">
         <v>7021</v>

</xml_diff>

<commit_message>
yerden2: Excel 17,5 W/m (şablon birim verimi), şema şap taraması, --etiket-ust
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RwXcqZmf9VPBpDgb8LPkn3
</commit_message>
<xml_diff>
--- a/proje/denemeler/yerden2/NB_YERDEN_ISITMA.xlsx
+++ b/proje/denemeler/yerden2/NB_YERDEN_ISITMA.xlsx
@@ -4700,7 +4700,7 @@
         </is>
       </c>
       <c r="D10" s="343" t="n">
-        <v>1604.4</v>
+        <v>802.2</v>
       </c>
       <c r="E10" s="344" t="n">
         <v>17.5</v>
@@ -4745,7 +4745,7 @@
         </is>
       </c>
       <c r="D11" s="343" t="n">
-        <v>2551.9</v>
+        <v>1275.9</v>
       </c>
       <c r="E11" s="344" t="n">
         <v>17.5</v>
@@ -4790,7 +4790,7 @@
         </is>
       </c>
       <c r="D12" s="343" t="n">
-        <v>1365.3</v>
+        <v>682.7</v>
       </c>
       <c r="E12" s="344" t="n">
         <v>17.5</v>
@@ -4835,7 +4835,7 @@
         </is>
       </c>
       <c r="D13" s="343" t="n">
-        <v>1544.2</v>
+        <v>772.1</v>
       </c>
       <c r="E13" s="344" t="n">
         <v>17.5</v>
@@ -4880,7 +4880,7 @@
         </is>
       </c>
       <c r="D14" s="343" t="n">
-        <v>3600.5</v>
+        <v>1800.2</v>
       </c>
       <c r="E14" s="344" t="n">
         <v>17.5</v>
@@ -4925,7 +4925,7 @@
         </is>
       </c>
       <c r="D15" s="343" t="n">
-        <v>1519.3</v>
+        <v>759.7</v>
       </c>
       <c r="E15" s="344" t="n">
         <v>17.5</v>
@@ -4970,7 +4970,7 @@
         </is>
       </c>
       <c r="D16" s="343" t="n">
-        <v>391.6</v>
+        <v>195.8</v>
       </c>
       <c r="E16" s="344" t="n">
         <v>17.5</v>
@@ -5015,7 +5015,7 @@
         </is>
       </c>
       <c r="D17" s="343" t="n">
-        <v>1694</v>
+        <v>847</v>
       </c>
       <c r="E17" s="344" t="n">
         <v>17.5</v>
@@ -5060,7 +5060,7 @@
         </is>
       </c>
       <c r="D18" s="343" t="n">
-        <v>2125.2</v>
+        <v>1062.6</v>
       </c>
       <c r="E18" s="344" t="n">
         <v>17.5</v>
@@ -5105,7 +5105,7 @@
         </is>
       </c>
       <c r="D19" s="343" t="n">
-        <v>1365.3</v>
+        <v>682.7</v>
       </c>
       <c r="E19" s="344" t="n">
         <v>17.5</v>
@@ -5150,7 +5150,7 @@
         </is>
       </c>
       <c r="D20" s="343" t="n">
-        <v>1481.9</v>
+        <v>741</v>
       </c>
       <c r="E20" s="344" t="n">
         <v>17.5</v>
@@ -5195,7 +5195,7 @@
         </is>
       </c>
       <c r="D21" s="343" t="n">
-        <v>3933.3</v>
+        <v>1966.6</v>
       </c>
       <c r="E21" s="344" t="n">
         <v>17.5</v>
@@ -5240,7 +5240,7 @@
         </is>
       </c>
       <c r="D22" s="343" t="n">
-        <v>1521.8</v>
+        <v>760.9</v>
       </c>
       <c r="E22" s="344" t="n">
         <v>17.5</v>
@@ -5285,7 +5285,7 @@
         </is>
       </c>
       <c r="D23" s="343" t="n">
-        <v>385.7</v>
+        <v>192.8</v>
       </c>
       <c r="E23" s="344" t="n">
         <v>17.5</v>
@@ -5330,7 +5330,7 @@
         </is>
       </c>
       <c r="D24" s="343" t="n">
-        <v>1006.6</v>
+        <v>503.3</v>
       </c>
       <c r="E24" s="344" t="n">
         <v>17.5</v>
@@ -5375,7 +5375,7 @@
         </is>
       </c>
       <c r="D25" s="348" t="n">
-        <v>2011</v>
+        <v>1005.5</v>
       </c>
       <c r="E25" s="349" t="n">
         <v>17.5</v>
@@ -5420,7 +5420,7 @@
         </is>
       </c>
       <c r="D26" s="348" t="n">
-        <v>1504.7</v>
+        <v>752.3</v>
       </c>
       <c r="E26" s="349" t="n">
         <v>17.5</v>
@@ -5465,7 +5465,7 @@
         </is>
       </c>
       <c r="D27" s="348" t="n">
-        <v>3407</v>
+        <v>1703.5</v>
       </c>
       <c r="E27" s="349" t="n">
         <v>17.5</v>
@@ -5510,7 +5510,7 @@
         </is>
       </c>
       <c r="D28" s="348" t="n">
-        <v>1254.4</v>
+        <v>627.2</v>
       </c>
       <c r="E28" s="349" t="n">
         <v>17.5</v>
@@ -5555,7 +5555,7 @@
         </is>
       </c>
       <c r="D29" s="348" t="n">
-        <v>1577.8</v>
+        <v>788.9</v>
       </c>
       <c r="E29" s="349" t="n">
         <v>17.5</v>
@@ -5600,7 +5600,7 @@
         </is>
       </c>
       <c r="D30" s="348" t="n">
-        <v>249.5</v>
+        <v>124.8</v>
       </c>
       <c r="E30" s="349" t="n">
         <v>17.5</v>
@@ -5678,7 +5678,7 @@
         </is>
       </c>
       <c r="D32" s="348" t="n">
-        <v>1695.4</v>
+        <v>847.7</v>
       </c>
       <c r="E32" s="349" t="n">
         <v>17.5</v>
@@ -5723,7 +5723,7 @@
         </is>
       </c>
       <c r="D33" s="348" t="n">
-        <v>2538.2</v>
+        <v>1269.1</v>
       </c>
       <c r="E33" s="349" t="n">
         <v>17.5</v>
@@ -5768,7 +5768,7 @@
         </is>
       </c>
       <c r="D34" s="348" t="n">
-        <v>1365.3</v>
+        <v>682.7</v>
       </c>
       <c r="E34" s="349" t="n">
         <v>17.5</v>
@@ -5813,7 +5813,7 @@
         </is>
       </c>
       <c r="D35" s="348" t="n">
-        <v>1481.9</v>
+        <v>741</v>
       </c>
       <c r="E35" s="349" t="n">
         <v>17.5</v>
@@ -5858,7 +5858,7 @@
         </is>
       </c>
       <c r="D36" s="348" t="n">
-        <v>3919.3</v>
+        <v>1959.7</v>
       </c>
       <c r="E36" s="349" t="n">
         <v>17.5</v>
@@ -5903,7 +5903,7 @@
         </is>
       </c>
       <c r="D37" s="348" t="n">
-        <v>1521.8</v>
+        <v>760.9</v>
       </c>
       <c r="E37" s="349" t="n">
         <v>17.5</v>
@@ -5948,7 +5948,7 @@
         </is>
       </c>
       <c r="D38" s="348" t="n">
-        <v>385</v>
+        <v>192.5</v>
       </c>
       <c r="E38" s="349" t="n">
         <v>17.5</v>
@@ -5993,7 +5993,7 @@
         </is>
       </c>
       <c r="D39" s="348" t="n">
-        <v>1176.7</v>
+        <v>588.3</v>
       </c>
       <c r="E39" s="349" t="n">
         <v>17.5</v>
@@ -6038,7 +6038,7 @@
         </is>
       </c>
       <c r="D40" s="348" t="n">
-        <v>2112.3</v>
+        <v>1056.1</v>
       </c>
       <c r="E40" s="349" t="n">
         <v>17.5</v>
@@ -6083,7 +6083,7 @@
         </is>
       </c>
       <c r="D41" s="348" t="n">
-        <v>1504.7</v>
+        <v>752.3</v>
       </c>
       <c r="E41" s="349" t="n">
         <v>17.5</v>
@@ -6128,7 +6128,7 @@
         </is>
       </c>
       <c r="D42" s="348" t="n">
-        <v>3226.3</v>
+        <v>1613.2</v>
       </c>
       <c r="E42" s="349" t="n">
         <v>17.5</v>
@@ -6173,7 +6173,7 @@
         </is>
       </c>
       <c r="D43" s="348" t="n">
-        <v>1086.8</v>
+        <v>543.4</v>
       </c>
       <c r="E43" s="349" t="n">
         <v>17.5</v>
@@ -6218,7 +6218,7 @@
         </is>
       </c>
       <c r="D44" s="348" t="n">
-        <v>1577.5</v>
+        <v>788.7</v>
       </c>
       <c r="E44" s="349" t="n">
         <v>17.5</v>
@@ -6263,7 +6263,7 @@
         </is>
       </c>
       <c r="D45" s="348" t="n">
-        <v>249.9</v>
+        <v>124.9</v>
       </c>
       <c r="E45" s="349" t="n">
         <v>17.5</v>
@@ -6308,7 +6308,7 @@
         </is>
       </c>
       <c r="D46" s="348" t="n">
-        <v>1688.4</v>
+        <v>844.2</v>
       </c>
       <c r="E46" s="349" t="n">
         <v>17.5</v>
@@ -6353,7 +6353,7 @@
         </is>
       </c>
       <c r="D47" s="348" t="n">
-        <v>2557.5</v>
+        <v>1278.7</v>
       </c>
       <c r="E47" s="349" t="n">
         <v>17.5</v>
@@ -6398,7 +6398,7 @@
         </is>
       </c>
       <c r="D48" s="348" t="n">
-        <v>1421.3</v>
+        <v>710.7</v>
       </c>
       <c r="E48" s="349" t="n">
         <v>17.5</v>
@@ -6443,7 +6443,7 @@
         </is>
       </c>
       <c r="D49" s="348" t="n">
-        <v>1499.4</v>
+        <v>749.7</v>
       </c>
       <c r="E49" s="349" t="n">
         <v>17.5</v>
@@ -6488,7 +6488,7 @@
         </is>
       </c>
       <c r="D50" s="348" t="n">
-        <v>3606.1</v>
+        <v>1803</v>
       </c>
       <c r="E50" s="349" t="n">
         <v>17.5</v>
@@ -6533,7 +6533,7 @@
         </is>
       </c>
       <c r="D51" s="348" t="n">
-        <v>1519.3</v>
+        <v>759.7</v>
       </c>
       <c r="E51" s="349" t="n">
         <v>17.5</v>
@@ -6578,7 +6578,7 @@
         </is>
       </c>
       <c r="D52" s="348" t="n">
-        <v>58.1</v>
+        <v>29</v>
       </c>
       <c r="E52" s="349" t="n">
         <v>17.5</v>
@@ -6623,7 +6623,7 @@
         </is>
       </c>
       <c r="D53" s="348" t="n">
-        <v>249.5</v>
+        <v>124.8</v>
       </c>
       <c r="E53" s="349" t="n">
         <v>17.5</v>
@@ -6701,7 +6701,7 @@
         </is>
       </c>
       <c r="D55" s="348" t="n">
-        <v>1586.9</v>
+        <v>793.5</v>
       </c>
       <c r="E55" s="349" t="n">
         <v>17.5</v>
@@ -6746,7 +6746,7 @@
         </is>
       </c>
       <c r="D56" s="348" t="n">
-        <v>2443.7</v>
+        <v>1221.8</v>
       </c>
       <c r="E56" s="349" t="n">
         <v>17.5</v>
@@ -6791,7 +6791,7 @@
         </is>
       </c>
       <c r="D57" s="348" t="n">
-        <v>1361.2</v>
+        <v>680.6</v>
       </c>
       <c r="E57" s="349" t="n">
         <v>17.5</v>
@@ -6836,7 +6836,7 @@
         </is>
       </c>
       <c r="D58" s="348" t="n">
-        <v>1490.3</v>
+        <v>745.1</v>
       </c>
       <c r="E58" s="349" t="n">
         <v>17.5</v>
@@ -6881,7 +6881,7 @@
         </is>
       </c>
       <c r="D59" s="348" t="n">
-        <v>3576.6</v>
+        <v>1788.3</v>
       </c>
       <c r="E59" s="349" t="n">
         <v>17.5</v>
@@ -6926,7 +6926,7 @@
         </is>
       </c>
       <c r="D60" s="348" t="n">
-        <v>1505.3</v>
+        <v>752.7</v>
       </c>
       <c r="E60" s="349" t="n">
         <v>17.5</v>
@@ -6971,7 +6971,7 @@
         </is>
       </c>
       <c r="D61" s="348" t="n">
-        <v>389.2</v>
+        <v>194.6</v>
       </c>
       <c r="E61" s="349" t="n">
         <v>17.5</v>
@@ -7016,7 +7016,7 @@
         </is>
       </c>
       <c r="D62" s="348" t="n">
-        <v>1189.3</v>
+        <v>594.6</v>
       </c>
       <c r="E62" s="349" t="n">
         <v>17.5</v>
@@ -7061,7 +7061,7 @@
         </is>
       </c>
       <c r="D63" s="348" t="n">
-        <v>1210.3</v>
+        <v>605.1</v>
       </c>
       <c r="E63" s="349" t="n">
         <v>17.5</v>
@@ -7106,7 +7106,7 @@
         </is>
       </c>
       <c r="D64" s="348" t="n">
-        <v>1539</v>
+        <v>769.5</v>
       </c>
       <c r="E64" s="349" t="n">
         <v>17.5</v>
@@ -7151,7 +7151,7 @@
         </is>
       </c>
       <c r="D65" s="348" t="n">
-        <v>2985.5</v>
+        <v>1492.8</v>
       </c>
       <c r="E65" s="349" t="n">
         <v>17.5</v>
@@ -7196,7 +7196,7 @@
         </is>
       </c>
       <c r="D66" s="348" t="n">
-        <v>1244.6</v>
+        <v>622.3</v>
       </c>
       <c r="E66" s="349" t="n">
         <v>17.5</v>
@@ -7241,7 +7241,7 @@
         </is>
       </c>
       <c r="D67" s="348" t="n">
-        <v>1575.7</v>
+        <v>787.9</v>
       </c>
       <c r="E67" s="349" t="n">
         <v>17.5</v>
@@ -7286,7 +7286,7 @@
         </is>
       </c>
       <c r="D68" s="348" t="n">
-        <v>247.5</v>
+        <v>123.7</v>
       </c>
       <c r="E68" s="349" t="n">
         <v>17.5</v>
@@ -7331,7 +7331,7 @@
         </is>
       </c>
       <c r="D69" s="348" t="n">
-        <v>1677.9</v>
+        <v>838.9</v>
       </c>
       <c r="E69" s="349" t="n">
         <v>17.5</v>
@@ -7376,7 +7376,7 @@
         </is>
       </c>
       <c r="D70" s="348" t="n">
-        <v>2544.2</v>
+        <v>1272.1</v>
       </c>
       <c r="E70" s="349" t="n">
         <v>17.5</v>
@@ -7421,7 +7421,7 @@
         </is>
       </c>
       <c r="D71" s="348" t="n">
-        <v>1372.4</v>
+        <v>686.2</v>
       </c>
       <c r="E71" s="349" t="n">
         <v>17.5</v>
@@ -7466,7 +7466,7 @@
         </is>
       </c>
       <c r="D72" s="348" t="n">
-        <v>1542.8</v>
+        <v>771.4</v>
       </c>
       <c r="E72" s="349" t="n">
         <v>17.5</v>
@@ -7511,7 +7511,7 @@
         </is>
       </c>
       <c r="D73" s="348" t="n">
-        <v>3559.8</v>
+        <v>1779.9</v>
       </c>
       <c r="E73" s="349" t="n">
         <v>17.5</v>
@@ -7556,7 +7556,7 @@
         </is>
       </c>
       <c r="D74" s="348" t="n">
-        <v>1505.7</v>
+        <v>752.9</v>
       </c>
       <c r="E74" s="349" t="n">
         <v>17.5</v>
@@ -7601,7 +7601,7 @@
         </is>
       </c>
       <c r="D75" s="348" t="n">
-        <v>362.6</v>
+        <v>181.3</v>
       </c>
       <c r="E75" s="349" t="n">
         <v>17.5</v>
@@ -13241,7 +13241,7 @@
       </c>
       <c r="E2" s="383" t="inlineStr">
         <is>
-          <t>TOPLAM ISI = 36095 W</t>
+          <t>TOPLAM ISI = 18048 W</t>
         </is>
       </c>
       <c r="F2" s="264" t="n"/>
@@ -13272,7 +13272,7 @@
       </c>
       <c r="E3" s="383" t="inlineStr">
         <is>
-          <t>MAX. BASINÇ KAYBI = 16935 Pa</t>
+          <t>MAX. BASINÇ KAYBI = 5035 Pa</t>
         </is>
       </c>
       <c r="F3" s="250" t="n"/>
@@ -14010,85 +14010,85 @@
       <c r="D13" s="261" t="n"/>
       <c r="E13" s="259" t="n"/>
       <c r="F13" s="398" t="n">
-        <v>1604.4</v>
+        <v>802.2</v>
       </c>
       <c r="G13" s="398" t="n">
-        <v>1180.9</v>
+        <v>590.5</v>
       </c>
       <c r="H13" s="398" t="n">
-        <v>1371</v>
+        <v>685.5</v>
       </c>
       <c r="I13" s="398" t="n">
-        <v>1365.3</v>
+        <v>682.7</v>
       </c>
       <c r="J13" s="398" t="n">
-        <v>1544.2</v>
+        <v>772.1</v>
       </c>
       <c r="K13" s="398" t="n">
-        <v>1749.7</v>
+        <v>874.8</v>
       </c>
       <c r="L13" s="398" t="n">
-        <v>1850.8</v>
+        <v>925.4</v>
       </c>
       <c r="M13" s="398" t="n">
-        <v>1519.3</v>
+        <v>759.7</v>
       </c>
       <c r="N13" s="398" t="n">
-        <v>391.6</v>
+        <v>195.8</v>
       </c>
       <c r="O13" s="398" t="n">
-        <v>1694</v>
+        <v>847</v>
       </c>
       <c r="P13" s="398" t="n">
-        <v>1091.3</v>
+        <v>545.6</v>
       </c>
       <c r="Q13" s="398" t="n">
-        <v>1033.9</v>
+        <v>516.9</v>
       </c>
       <c r="R13" s="398" t="n">
-        <v>1365.3</v>
+        <v>682.7</v>
       </c>
       <c r="S13" s="398" t="n">
-        <v>1481.9</v>
+        <v>741</v>
       </c>
       <c r="T13" s="398" t="n">
-        <v>2082.5</v>
+        <v>1041.2</v>
       </c>
       <c r="U13" s="398" t="n">
-        <v>1850.8</v>
+        <v>925.4</v>
       </c>
       <c r="V13" s="398" t="n">
-        <v>1521.8</v>
+        <v>760.9</v>
       </c>
       <c r="W13" s="398" t="n">
-        <v>385.7</v>
+        <v>192.8</v>
       </c>
       <c r="X13" s="398" t="n">
-        <v>1006.6</v>
+        <v>503.3</v>
       </c>
       <c r="Y13" s="398" t="n">
-        <v>949.5</v>
+        <v>474.8</v>
       </c>
       <c r="Z13" s="398" t="n">
-        <v>1061.5</v>
+        <v>530.8</v>
       </c>
       <c r="AA13" s="398" t="n">
-        <v>1504.7</v>
+        <v>752.3</v>
       </c>
       <c r="AB13" s="398" t="n">
-        <v>1808.5</v>
+        <v>904.2</v>
       </c>
       <c r="AC13" s="398" t="n">
-        <v>1598.5</v>
+        <v>799.2</v>
       </c>
       <c r="AD13" s="398" t="n">
-        <v>1254.4</v>
+        <v>627.2</v>
       </c>
       <c r="AE13" s="398" t="n">
-        <v>1577.8</v>
+        <v>788.9</v>
       </c>
       <c r="AF13" s="398" t="n">
-        <v>249.5</v>
+        <v>124.8</v>
       </c>
     </row>
     <row r="14" ht="12" customHeight="1" s="244">
@@ -16022,85 +16022,85 @@
       </c>
       <c r="E32" s="259" t="n"/>
       <c r="F32" s="407" t="n">
-        <v>7872</v>
+        <v>2340</v>
       </c>
       <c r="G32" s="407" t="n">
-        <v>3389</v>
+        <v>615</v>
       </c>
       <c r="H32" s="407" t="n">
-        <v>5109</v>
+        <v>1519</v>
       </c>
       <c r="I32" s="407" t="n">
-        <v>5051</v>
+        <v>1502</v>
       </c>
       <c r="J32" s="407" t="n">
-        <v>7087</v>
+        <v>2107</v>
       </c>
       <c r="K32" s="407" t="n">
-        <v>9992</v>
+        <v>2970</v>
       </c>
       <c r="L32" s="407" t="n">
-        <v>11661</v>
+        <v>3467</v>
       </c>
       <c r="M32" s="407" t="n">
-        <v>6777</v>
+        <v>2015</v>
       </c>
       <c r="N32" s="407" t="n">
-        <v>135</v>
+        <v>68</v>
       </c>
       <c r="O32" s="407" t="n">
-        <v>9141</v>
+        <v>2718</v>
       </c>
       <c r="P32" s="407" t="n">
-        <v>2728</v>
+        <v>525</v>
       </c>
       <c r="Q32" s="407" t="n">
-        <v>2351</v>
+        <v>472</v>
       </c>
       <c r="R32" s="407" t="n">
-        <v>5051</v>
+        <v>1502</v>
       </c>
       <c r="S32" s="407" t="n">
-        <v>6328</v>
+        <v>1881</v>
       </c>
       <c r="T32" s="407" t="n">
-        <v>16129</v>
+        <v>4795</v>
       </c>
       <c r="U32" s="407" t="n">
-        <v>11661</v>
+        <v>3467</v>
       </c>
       <c r="V32" s="407" t="n">
-        <v>6807</v>
+        <v>2024</v>
       </c>
       <c r="W32" s="407" t="n">
-        <v>131</v>
+        <v>66</v>
       </c>
       <c r="X32" s="407" t="n">
-        <v>2185</v>
+        <v>447</v>
       </c>
       <c r="Y32" s="407" t="n">
-        <v>1861</v>
+        <v>398</v>
       </c>
       <c r="Z32" s="407" t="n">
-        <v>2528</v>
+        <v>497</v>
       </c>
       <c r="AA32" s="407" t="n">
-        <v>6599</v>
+        <v>1962</v>
       </c>
       <c r="AB32" s="407" t="n">
-        <v>10942</v>
+        <v>3253</v>
       </c>
       <c r="AC32" s="407" t="n">
-        <v>7793</v>
+        <v>2317</v>
       </c>
       <c r="AD32" s="407" t="n">
-        <v>4001</v>
+        <v>1190</v>
       </c>
       <c r="AE32" s="407" t="n">
-        <v>7519</v>
+        <v>2235</v>
       </c>
       <c r="AF32" s="407" t="n">
-        <v>55</v>
+        <v>27</v>
       </c>
     </row>
     <row r="33" ht="12" customHeight="1" s="244">
@@ -16535,7 +16535,7 @@
       </c>
       <c r="B43" s="243" t="inlineStr">
         <is>
-          <t>Alta geçen ısı 0,2 q" olarak alınmıştır.</t>
+          <t>Alta geçen ısı 0,2 q" olarak alınmıştır. qh = 17,5 W/m × devre boyu (şablon birim verimi); ısı kaybı hesabı ayrıca yapılmalıdır.</t>
         </is>
       </c>
     </row>
@@ -16671,7 +16671,7 @@
       </c>
       <c r="E2" s="383" t="inlineStr">
         <is>
-          <t>TOPLAM ISI = 36441 W</t>
+          <t>TOPLAM ISI = 18220 W</t>
         </is>
       </c>
       <c r="F2" s="264" t="n"/>
@@ -16710,7 +16710,7 @@
       </c>
       <c r="E3" s="383" t="inlineStr">
         <is>
-          <t>MAX. BASINÇ KAYBI = 16624 Pa</t>
+          <t>MAX. BASINÇ KAYBI = 4942 Pa</t>
         </is>
       </c>
       <c r="F3" s="250" t="n"/>
@@ -17585,88 +17585,88 @@
       <c r="D13" s="261" t="n"/>
       <c r="E13" s="259" t="n"/>
       <c r="F13" s="398" t="n">
-        <v>1695.4</v>
+        <v>847.7</v>
       </c>
       <c r="G13" s="398" t="n">
-        <v>1480.5</v>
+        <v>740.2</v>
       </c>
       <c r="H13" s="398" t="n">
-        <v>1057.7</v>
+        <v>528.9</v>
       </c>
       <c r="I13" s="398" t="n">
-        <v>1365.3</v>
+        <v>682.7</v>
       </c>
       <c r="J13" s="398" t="n">
-        <v>1481.9</v>
+        <v>741</v>
       </c>
       <c r="K13" s="398" t="n">
-        <v>2068.5</v>
+        <v>1034.2</v>
       </c>
       <c r="L13" s="398" t="n">
-        <v>1850.8</v>
+        <v>925.4</v>
       </c>
       <c r="M13" s="398" t="n">
-        <v>1521.8</v>
+        <v>760.9</v>
       </c>
       <c r="N13" s="398" t="n">
-        <v>385</v>
+        <v>192.5</v>
       </c>
       <c r="O13" s="398" t="n">
-        <v>1176.7</v>
+        <v>588.3</v>
       </c>
       <c r="P13" s="398" t="n">
-        <v>981.8</v>
+        <v>490.9</v>
       </c>
       <c r="Q13" s="398" t="n">
-        <v>1130.5</v>
+        <v>565.2</v>
       </c>
       <c r="R13" s="398" t="n">
-        <v>1504.7</v>
+        <v>752.3</v>
       </c>
       <c r="S13" s="398" t="n">
-        <v>1708</v>
+        <v>854</v>
       </c>
       <c r="T13" s="398" t="n">
-        <v>1518.3</v>
+        <v>759.2</v>
       </c>
       <c r="U13" s="398" t="n">
-        <v>1086.8</v>
+        <v>543.4</v>
       </c>
       <c r="V13" s="398" t="n">
-        <v>1577.5</v>
+        <v>788.7</v>
       </c>
       <c r="W13" s="398" t="n">
-        <v>249.9</v>
+        <v>124.9</v>
       </c>
       <c r="X13" s="398" t="n">
-        <v>1688.4</v>
+        <v>844.2</v>
       </c>
       <c r="Y13" s="398" t="n">
-        <v>1185.1</v>
+        <v>592.5</v>
       </c>
       <c r="Z13" s="398" t="n">
-        <v>1372.4</v>
+        <v>686.2</v>
       </c>
       <c r="AA13" s="398" t="n">
-        <v>1421.3</v>
+        <v>710.7</v>
       </c>
       <c r="AB13" s="398" t="n">
-        <v>1499.4</v>
+        <v>749.7</v>
       </c>
       <c r="AC13" s="398" t="n">
-        <v>1752.5</v>
+        <v>876.2</v>
       </c>
       <c r="AD13" s="398" t="n">
-        <v>1853.6</v>
+        <v>926.8</v>
       </c>
       <c r="AE13" s="398" t="n">
-        <v>1519.3</v>
+        <v>759.7</v>
       </c>
       <c r="AF13" s="398" t="n">
-        <v>58.1</v>
+        <v>29</v>
       </c>
       <c r="AG13" s="398" t="n">
-        <v>249.5</v>
+        <v>124.8</v>
       </c>
       <c r="AH13" s="425" t="n"/>
       <c r="AI13" s="425" t="n"/>
@@ -19963,88 +19963,88 @@
       </c>
       <c r="E32" s="259" t="n"/>
       <c r="F32" s="407" t="n">
-        <v>9162</v>
+        <v>2724</v>
       </c>
       <c r="G32" s="407" t="n">
-        <v>6311</v>
+        <v>1876</v>
       </c>
       <c r="H32" s="407" t="n">
-        <v>2503</v>
+        <v>494</v>
       </c>
       <c r="I32" s="407" t="n">
-        <v>5051</v>
+        <v>1502</v>
       </c>
       <c r="J32" s="407" t="n">
-        <v>6328</v>
+        <v>1881</v>
       </c>
       <c r="K32" s="407" t="n">
-        <v>15833</v>
+        <v>4707</v>
       </c>
       <c r="L32" s="407" t="n">
-        <v>11661</v>
+        <v>3467</v>
       </c>
       <c r="M32" s="407" t="n">
-        <v>6807</v>
+        <v>2024</v>
       </c>
       <c r="N32" s="407" t="n">
-        <v>131</v>
+        <v>65</v>
       </c>
       <c r="O32" s="407" t="n">
-        <v>3356</v>
+        <v>611</v>
       </c>
       <c r="P32" s="407" t="n">
-        <v>2040</v>
+        <v>425</v>
       </c>
       <c r="Q32" s="407" t="n">
-        <v>3006</v>
+        <v>564</v>
       </c>
       <c r="R32" s="407" t="n">
-        <v>6599</v>
+        <v>1962</v>
       </c>
       <c r="S32" s="407" t="n">
-        <v>9351</v>
+        <v>2780</v>
       </c>
       <c r="T32" s="407" t="n">
-        <v>6764</v>
+        <v>2011</v>
       </c>
       <c r="U32" s="407" t="n">
-        <v>2697</v>
+        <v>521</v>
       </c>
       <c r="V32" s="407" t="n">
-        <v>7515</v>
+        <v>2234</v>
       </c>
       <c r="W32" s="407" t="n">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="X32" s="407" t="n">
-        <v>9058</v>
+        <v>2693</v>
       </c>
       <c r="Y32" s="407" t="n">
-        <v>3422</v>
+        <v>1017</v>
       </c>
       <c r="Z32" s="407" t="n">
-        <v>5123</v>
+        <v>1523</v>
       </c>
       <c r="AA32" s="407" t="n">
-        <v>5642</v>
+        <v>1677</v>
       </c>
       <c r="AB32" s="407" t="n">
-        <v>6535</v>
+        <v>1943</v>
       </c>
       <c r="AC32" s="407" t="n">
-        <v>10036</v>
+        <v>2983</v>
       </c>
       <c r="AD32" s="407" t="n">
-        <v>11710</v>
+        <v>3481</v>
       </c>
       <c r="AE32" s="407" t="n">
-        <v>6777</v>
+        <v>2015</v>
       </c>
       <c r="AF32" s="407" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AG32" s="407" t="n">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="AH32" s="431" t="n"/>
       <c r="AI32" s="431" t="n"/>
@@ -20568,7 +20568,7 @@
       </c>
       <c r="B43" s="243" t="inlineStr">
         <is>
-          <t>Alta geçen ısı 0,2 q" olarak alınmıştır.</t>
+          <t>Alta geçen ısı 0,2 q" olarak alınmıştır. qh = 17,5 W/m × devre boyu (şablon birim verimi); ısı kaybı hesabı ayrıca yapılmalıdır.</t>
         </is>
       </c>
     </row>
@@ -20704,7 +20704,7 @@
       </c>
       <c r="E2" s="383" t="inlineStr">
         <is>
-          <t>TOPLAM ISI = 34910 W</t>
+          <t>TOPLAM ISI = 17455 W</t>
         </is>
       </c>
       <c r="F2" s="264" t="n"/>
@@ -20743,7 +20743,7 @@
       </c>
       <c r="E3" s="383" t="inlineStr">
         <is>
-          <t>MAX. BASINÇ KAYBI = 12168 Pa</t>
+          <t>MAX. BASINÇ KAYBI = 3618 Pa</t>
         </is>
       </c>
       <c r="F3" s="250" t="n"/>
@@ -21602,85 +21602,85 @@
       <c r="D13" s="261" t="n"/>
       <c r="E13" s="259" t="n"/>
       <c r="F13" s="398" t="n">
-        <v>1586.9</v>
+        <v>793.5</v>
       </c>
       <c r="G13" s="398" t="n">
-        <v>1100</v>
+        <v>550</v>
       </c>
       <c r="H13" s="398" t="n">
-        <v>1343.7</v>
+        <v>671.8</v>
       </c>
       <c r="I13" s="398" t="n">
-        <v>1361.2</v>
+        <v>680.6</v>
       </c>
       <c r="J13" s="398" t="n">
-        <v>1490.3</v>
+        <v>745.1</v>
       </c>
       <c r="K13" s="398" t="n">
-        <v>1730</v>
+        <v>865</v>
       </c>
       <c r="L13" s="398" t="n">
-        <v>1846.6</v>
+        <v>923.3</v>
       </c>
       <c r="M13" s="398" t="n">
-        <v>1505.3</v>
+        <v>752.7</v>
       </c>
       <c r="N13" s="398" t="n">
-        <v>389.2</v>
+        <v>194.6</v>
       </c>
       <c r="O13" s="398" t="n">
-        <v>1189.3</v>
+        <v>594.6</v>
       </c>
       <c r="P13" s="398" t="n">
-        <v>583.1</v>
+        <v>291.6</v>
       </c>
       <c r="Q13" s="398" t="n">
-        <v>627.2</v>
+        <v>313.6</v>
       </c>
       <c r="R13" s="398" t="n">
-        <v>1539</v>
+        <v>769.5</v>
       </c>
       <c r="S13" s="398" t="n">
-        <v>1571.2</v>
+        <v>785.6</v>
       </c>
       <c r="T13" s="398" t="n">
-        <v>1414.3</v>
+        <v>707.2</v>
       </c>
       <c r="U13" s="398" t="n">
-        <v>1244.6</v>
+        <v>622.3</v>
       </c>
       <c r="V13" s="398" t="n">
-        <v>1575.7</v>
+        <v>787.9</v>
       </c>
       <c r="W13" s="398" t="n">
-        <v>247.5</v>
+        <v>123.7</v>
       </c>
       <c r="X13" s="398" t="n">
-        <v>1677.9</v>
+        <v>838.9</v>
       </c>
       <c r="Y13" s="398" t="n">
-        <v>1177.8</v>
+        <v>588.9</v>
       </c>
       <c r="Z13" s="398" t="n">
-        <v>1366.4</v>
+        <v>683.2</v>
       </c>
       <c r="AA13" s="398" t="n">
-        <v>1372.4</v>
+        <v>686.2</v>
       </c>
       <c r="AB13" s="398" t="n">
-        <v>1542.8</v>
+        <v>771.4</v>
       </c>
       <c r="AC13" s="398" t="n">
-        <v>1713.2</v>
+        <v>856.6</v>
       </c>
       <c r="AD13" s="398" t="n">
-        <v>1846.6</v>
+        <v>923.3</v>
       </c>
       <c r="AE13" s="398" t="n">
-        <v>1505.7</v>
+        <v>752.9</v>
       </c>
       <c r="AF13" s="398" t="n">
-        <v>362.6</v>
+        <v>181.3</v>
       </c>
       <c r="AG13" s="425" t="n"/>
       <c r="AH13" s="425" t="n"/>
@@ -23930,85 +23930,85 @@
       </c>
       <c r="E32" s="259" t="n"/>
       <c r="F32" s="407" t="n">
-        <v>7639</v>
+        <v>2271</v>
       </c>
       <c r="G32" s="407" t="n">
-        <v>2788</v>
+        <v>534</v>
       </c>
       <c r="H32" s="407" t="n">
-        <v>4834</v>
+        <v>1437</v>
       </c>
       <c r="I32" s="407" t="n">
-        <v>5009</v>
+        <v>1489</v>
       </c>
       <c r="J32" s="407" t="n">
-        <v>6427</v>
+        <v>1911</v>
       </c>
       <c r="K32" s="407" t="n">
-        <v>9686</v>
+        <v>2880</v>
       </c>
       <c r="L32" s="407" t="n">
-        <v>11588</v>
+        <v>3445</v>
       </c>
       <c r="M32" s="407" t="n">
-        <v>6607</v>
+        <v>1964</v>
       </c>
       <c r="N32" s="407" t="n">
-        <v>134</v>
+        <v>67</v>
       </c>
       <c r="O32" s="407" t="n">
-        <v>3456</v>
+        <v>1027</v>
       </c>
       <c r="P32" s="407" t="n">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="Q32" s="407" t="n">
-        <v>595</v>
+        <v>174</v>
       </c>
       <c r="R32" s="407" t="n">
-        <v>7021</v>
+        <v>2087</v>
       </c>
       <c r="S32" s="407" t="n">
-        <v>7432</v>
+        <v>2210</v>
       </c>
       <c r="T32" s="407" t="n">
-        <v>5565</v>
+        <v>1655</v>
       </c>
       <c r="U32" s="407" t="n">
-        <v>3916</v>
+        <v>1164</v>
       </c>
       <c r="V32" s="407" t="n">
-        <v>7491</v>
+        <v>2227</v>
       </c>
       <c r="W32" s="407" t="n">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="X32" s="407" t="n">
-        <v>8904</v>
+        <v>2647</v>
       </c>
       <c r="Y32" s="407" t="n">
-        <v>3365</v>
+        <v>612</v>
       </c>
       <c r="Z32" s="407" t="n">
-        <v>5062</v>
+        <v>1505</v>
       </c>
       <c r="AA32" s="407" t="n">
-        <v>5123</v>
+        <v>1523</v>
       </c>
       <c r="AB32" s="407" t="n">
-        <v>7069</v>
+        <v>2102</v>
       </c>
       <c r="AC32" s="407" t="n">
-        <v>9429</v>
+        <v>2804</v>
       </c>
       <c r="AD32" s="407" t="n">
-        <v>11588</v>
+        <v>3445</v>
       </c>
       <c r="AE32" s="407" t="n">
-        <v>6611</v>
+        <v>1966</v>
       </c>
       <c r="AF32" s="407" t="n">
-        <v>116</v>
+        <v>58</v>
       </c>
       <c r="AG32" s="431" t="n"/>
       <c r="AH32" s="431" t="n"/>
@@ -24524,7 +24524,7 @@
       </c>
       <c r="B43" s="243" t="inlineStr">
         <is>
-          <t>Alta geçen ısı 0,2 q" olarak alınmıştır.</t>
+          <t>Alta geçen ısı 0,2 q" olarak alınmıştır. qh = 17,5 W/m × devre boyu (şablon birim verimi); ısı kaybı hesabı ayrıca yapılmalıdır.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
yerden2: köşe girintisinde alt satır atlama, dış etiket puanlama
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RwXcqZmf9VPBpDgb8LPkn3
</commit_message>
<xml_diff>
--- a/proje/denemeler/yerden2/NB_YERDEN_ISITMA.xlsx
+++ b/proje/denemeler/yerden2/NB_YERDEN_ISITMA.xlsx
@@ -4970,7 +4970,7 @@
         </is>
       </c>
       <c r="D16" s="343" t="n">
-        <v>195.8</v>
+        <v>232.6</v>
       </c>
       <c r="E16" s="344" t="n">
         <v>17.5</v>
@@ -4980,7 +4980,7 @@
         <v/>
       </c>
       <c r="G16" s="340" t="n">
-        <v>11.19</v>
+        <v>13.29</v>
       </c>
       <c r="H16" s="340" t="n">
         <v>1</v>
@@ -5060,7 +5060,7 @@
         </is>
       </c>
       <c r="D18" s="343" t="n">
-        <v>1062.6</v>
+        <v>1222.7</v>
       </c>
       <c r="E18" s="344" t="n">
         <v>17.5</v>
@@ -5070,7 +5070,7 @@
         <v/>
       </c>
       <c r="G18" s="340" t="n">
-        <v>60.72</v>
+        <v>69.87</v>
       </c>
       <c r="H18" s="340" t="n">
         <v>2</v>
@@ -5330,7 +5330,7 @@
         </is>
       </c>
       <c r="D24" s="343" t="n">
-        <v>503.3</v>
+        <v>589</v>
       </c>
       <c r="E24" s="344" t="n">
         <v>17.5</v>
@@ -5340,7 +5340,7 @@
         <v/>
       </c>
       <c r="G24" s="340" t="n">
-        <v>28.76</v>
+        <v>33.66</v>
       </c>
       <c r="H24" s="340" t="n">
         <v>1</v>
@@ -6971,7 +6971,7 @@
         </is>
       </c>
       <c r="D61" s="348" t="n">
-        <v>194.6</v>
+        <v>211.4</v>
       </c>
       <c r="E61" s="349" t="n">
         <v>17.5</v>
@@ -6981,7 +6981,7 @@
         <v/>
       </c>
       <c r="G61" s="345" t="n">
-        <v>11.12</v>
+        <v>12.08</v>
       </c>
       <c r="H61" s="345" t="n">
         <v>1</v>
@@ -7061,7 +7061,7 @@
         </is>
       </c>
       <c r="D63" s="348" t="n">
-        <v>605.1</v>
+        <v>932.2</v>
       </c>
       <c r="E63" s="349" t="n">
         <v>17.5</v>
@@ -7071,7 +7071,7 @@
         <v/>
       </c>
       <c r="G63" s="345" t="n">
-        <v>34.58</v>
+        <v>53.27</v>
       </c>
       <c r="H63" s="345" t="n">
         <v>2</v>
@@ -7601,7 +7601,7 @@
         </is>
       </c>
       <c r="D75" s="348" t="n">
-        <v>181.3</v>
+        <v>233.4</v>
       </c>
       <c r="E75" s="349" t="n">
         <v>17.5</v>
@@ -7611,7 +7611,7 @@
         <v/>
       </c>
       <c r="G75" s="345" t="n">
-        <v>10.36</v>
+        <v>13.34</v>
       </c>
       <c r="H75" s="345" t="n">
         <v>1</v>
@@ -13241,7 +13241,7 @@
       </c>
       <c r="E2" s="383" t="inlineStr">
         <is>
-          <t>TOPLAM ISI = 18048 W</t>
+          <t>TOPLAM ISI = 18330 W</t>
         </is>
       </c>
       <c r="F2" s="264" t="n"/>
@@ -13952,10 +13952,10 @@
         <v>7.87</v>
       </c>
       <c r="P12" s="397" t="n">
-        <v>6.92</v>
+        <v>6.27</v>
       </c>
       <c r="Q12" s="397" t="n">
-        <v>6.55</v>
+        <v>7.2</v>
       </c>
       <c r="R12" s="397" t="n">
         <v>8.73</v>
@@ -14034,16 +14034,16 @@
         <v>759.7</v>
       </c>
       <c r="N13" s="398" t="n">
-        <v>195.8</v>
+        <v>232.6</v>
       </c>
       <c r="O13" s="398" t="n">
         <v>847</v>
       </c>
       <c r="P13" s="398" t="n">
-        <v>545.6</v>
+        <v>569.3</v>
       </c>
       <c r="Q13" s="398" t="n">
-        <v>516.9</v>
+        <v>653.5</v>
       </c>
       <c r="R13" s="398" t="n">
         <v>682.7</v>
@@ -14064,7 +14064,7 @@
         <v>192.8</v>
       </c>
       <c r="X13" s="398" t="n">
-        <v>503.3</v>
+        <v>589</v>
       </c>
       <c r="Y13" s="398" t="n">
         <v>474.8</v>
@@ -16046,16 +16046,16 @@
         <v>2015</v>
       </c>
       <c r="N32" s="407" t="n">
-        <v>68</v>
+        <v>95</v>
       </c>
       <c r="O32" s="407" t="n">
         <v>2718</v>
       </c>
       <c r="P32" s="407" t="n">
-        <v>525</v>
+        <v>572</v>
       </c>
       <c r="Q32" s="407" t="n">
-        <v>472</v>
+        <v>1332</v>
       </c>
       <c r="R32" s="407" t="n">
         <v>1502</v>
@@ -16076,7 +16076,7 @@
         <v>66</v>
       </c>
       <c r="X32" s="407" t="n">
-        <v>447</v>
+        <v>612</v>
       </c>
       <c r="Y32" s="407" t="n">
         <v>398</v>
@@ -20704,7 +20704,7 @@
       </c>
       <c r="E2" s="383" t="inlineStr">
         <is>
-          <t>TOPLAM ISI = 17455 W</t>
+          <t>TOPLAM ISI = 17851 W</t>
         </is>
       </c>
       <c r="F2" s="264" t="n"/>
@@ -21527,10 +21527,10 @@
         <v>6.92</v>
       </c>
       <c r="P12" s="397" t="n">
-        <v>6.75</v>
+        <v>7.39</v>
       </c>
       <c r="Q12" s="397" t="n">
-        <v>7.27</v>
+        <v>6.63</v>
       </c>
       <c r="R12" s="397" t="n">
         <v>8.66</v>
@@ -21626,16 +21626,16 @@
         <v>752.7</v>
       </c>
       <c r="N13" s="398" t="n">
-        <v>194.6</v>
+        <v>211.4</v>
       </c>
       <c r="O13" s="398" t="n">
         <v>594.6</v>
       </c>
       <c r="P13" s="398" t="n">
-        <v>291.6</v>
+        <v>491.6</v>
       </c>
       <c r="Q13" s="398" t="n">
-        <v>313.6</v>
+        <v>440.6</v>
       </c>
       <c r="R13" s="398" t="n">
         <v>769.5</v>
@@ -21680,7 +21680,7 @@
         <v>752.9</v>
       </c>
       <c r="AF13" s="398" t="n">
-        <v>181.3</v>
+        <v>233.4</v>
       </c>
       <c r="AG13" s="425" t="n"/>
       <c r="AH13" s="425" t="n"/>
@@ -23954,16 +23954,16 @@
         <v>1964</v>
       </c>
       <c r="N32" s="407" t="n">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="O32" s="407" t="n">
         <v>1027</v>
       </c>
       <c r="P32" s="407" t="n">
-        <v>150</v>
+        <v>426</v>
       </c>
       <c r="Q32" s="407" t="n">
-        <v>174</v>
+        <v>343</v>
       </c>
       <c r="R32" s="407" t="n">
         <v>2087</v>
@@ -24008,7 +24008,7 @@
         <v>1966</v>
       </c>
       <c r="AF32" s="407" t="n">
-        <v>58</v>
+        <v>96</v>
       </c>
       <c r="AG32" s="431" t="n"/>
       <c r="AH32" s="431" t="n"/>

</xml_diff>

<commit_message>
yerden2 tur 3 (ara): yüklük yarı düzlem kesitiyle ayrılıyor (Y-1, 3 katta), ıslak hacimde Ç.M. hariç + vitrifiye payı daraltıldı + gerekirse 6/5 cm duvar payı (Y-2), iki devreli mahalde etiket kendi bandında (Y-3), etiket önce çizgisiz serbest zeminde, çizgi üstündeyse kesik maske (Y-4)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RwXcqZmf9VPBpDgb8LPkn3
</commit_message>
<xml_diff>
--- a/proje/denemeler/yerden2/NB_YERDEN_ISITMA.xlsx
+++ b/proje/denemeler/yerden2/NB_YERDEN_ISITMA.xlsx
@@ -4652,7 +4652,7 @@
         </is>
       </c>
       <c r="D16" s="343" t="n">
-        <v>596.1</v>
+        <v>602.4</v>
       </c>
       <c r="E16" s="344" t="n">
         <v>35</v>
@@ -4662,7 +4662,7 @@
         <v/>
       </c>
       <c r="G16" s="340" t="n">
-        <v>17.03</v>
+        <v>17.21</v>
       </c>
       <c r="H16" s="340" t="n">
         <v>1</v>
@@ -4742,7 +4742,7 @@
         </is>
       </c>
       <c r="D18" s="343" t="n">
-        <v>2845.1</v>
+        <v>2889.9</v>
       </c>
       <c r="E18" s="344" t="n">
         <v>35</v>
@@ -4752,7 +4752,7 @@
         <v/>
       </c>
       <c r="G18" s="340" t="n">
-        <v>81.29000000000001</v>
+        <v>82.56999999999999</v>
       </c>
       <c r="H18" s="340" t="n">
         <v>2</v>
@@ -4967,7 +4967,7 @@
         </is>
       </c>
       <c r="D23" s="343" t="n">
-        <v>561.1</v>
+        <v>611.4</v>
       </c>
       <c r="E23" s="344" t="n">
         <v>35</v>
@@ -4977,7 +4977,7 @@
         <v/>
       </c>
       <c r="G23" s="340" t="n">
-        <v>16.03</v>
+        <v>17.47</v>
       </c>
       <c r="H23" s="340" t="n">
         <v>1</v>
@@ -5282,7 +5282,7 @@
         </is>
       </c>
       <c r="D30" s="348" t="n">
-        <v>419.7</v>
+        <v>349</v>
       </c>
       <c r="E30" s="349" t="n">
         <v>35</v>
@@ -5292,7 +5292,7 @@
         <v/>
       </c>
       <c r="G30" s="345" t="n">
-        <v>11.99</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="H30" s="345" t="n">
         <v>1</v>
@@ -5405,7 +5405,7 @@
         </is>
       </c>
       <c r="D33" s="348" t="n">
-        <v>3069.5</v>
+        <v>2889.9</v>
       </c>
       <c r="E33" s="349" t="n">
         <v>35</v>
@@ -5415,7 +5415,7 @@
         <v/>
       </c>
       <c r="G33" s="345" t="n">
-        <v>87.7</v>
+        <v>82.56999999999999</v>
       </c>
       <c r="H33" s="345" t="n">
         <v>2</v>
@@ -5630,7 +5630,7 @@
         </is>
       </c>
       <c r="D38" s="348" t="n">
-        <v>560.7</v>
+        <v>582</v>
       </c>
       <c r="E38" s="349" t="n">
         <v>35</v>
@@ -5640,7 +5640,7 @@
         <v/>
       </c>
       <c r="G38" s="345" t="n">
-        <v>16.02</v>
+        <v>16.63</v>
       </c>
       <c r="H38" s="345" t="n">
         <v>1</v>
@@ -5945,7 +5945,7 @@
         </is>
       </c>
       <c r="D45" s="348" t="n">
-        <v>419.7</v>
+        <v>349.3</v>
       </c>
       <c r="E45" s="349" t="n">
         <v>35</v>
@@ -5955,7 +5955,7 @@
         <v/>
       </c>
       <c r="G45" s="345" t="n">
-        <v>11.99</v>
+        <v>9.98</v>
       </c>
       <c r="H45" s="345" t="n">
         <v>1</v>
@@ -6260,7 +6260,7 @@
         </is>
       </c>
       <c r="D52" s="348" t="n">
-        <v>425.9</v>
+        <v>524.6</v>
       </c>
       <c r="E52" s="349" t="n">
         <v>35</v>
@@ -6270,7 +6270,7 @@
         <v/>
       </c>
       <c r="G52" s="345" t="n">
-        <v>12.17</v>
+        <v>14.99</v>
       </c>
       <c r="H52" s="345" t="n">
         <v>1</v>
@@ -6383,7 +6383,7 @@
         </is>
       </c>
       <c r="D55" s="348" t="n">
-        <v>3057.2</v>
+        <v>2867.2</v>
       </c>
       <c r="E55" s="349" t="n">
         <v>35</v>
@@ -6393,7 +6393,7 @@
         <v/>
       </c>
       <c r="G55" s="345" t="n">
-        <v>87.34999999999999</v>
+        <v>81.92</v>
       </c>
       <c r="H55" s="345" t="n">
         <v>2</v>
@@ -6608,7 +6608,7 @@
         </is>
       </c>
       <c r="D60" s="348" t="n">
-        <v>621.2</v>
+        <v>627.5</v>
       </c>
       <c r="E60" s="349" t="n">
         <v>35</v>
@@ -6618,7 +6618,7 @@
         <v/>
       </c>
       <c r="G60" s="345" t="n">
-        <v>17.75</v>
+        <v>17.93</v>
       </c>
       <c r="H60" s="345" t="n">
         <v>1</v>
@@ -6923,7 +6923,7 @@
         </is>
       </c>
       <c r="D67" s="348" t="n">
-        <v>420.3</v>
+        <v>344.1</v>
       </c>
       <c r="E67" s="349" t="n">
         <v>35</v>
@@ -6933,7 +6933,7 @@
         <v/>
       </c>
       <c r="G67" s="345" t="n">
-        <v>12.01</v>
+        <v>9.83</v>
       </c>
       <c r="H67" s="345" t="n">
         <v>1</v>
@@ -7238,7 +7238,7 @@
         </is>
       </c>
       <c r="D74" s="348" t="n">
-        <v>627.5</v>
+        <v>646.8</v>
       </c>
       <c r="E74" s="349" t="n">
         <v>35</v>
@@ -7248,7 +7248,7 @@
         <v/>
       </c>
       <c r="G74" s="345" t="n">
-        <v>17.93</v>
+        <v>18.48</v>
       </c>
       <c r="H74" s="345" t="n">
         <v>1</v>
@@ -12824,7 +12824,7 @@
       </c>
       <c r="E2" s="383" t="inlineStr">
         <is>
-          <t>TOPLAM ISI = 43972 W</t>
+          <t>TOPLAM ISI = 44002 W</t>
         </is>
       </c>
       <c r="F2" s="264" t="n"/>
@@ -13529,16 +13529,16 @@
         <v>7.61</v>
       </c>
       <c r="N12" s="397" t="n">
-        <v>3.38</v>
+        <v>3.39</v>
       </c>
       <c r="O12" s="397" t="n">
         <v>7.87</v>
       </c>
       <c r="P12" s="397" t="n">
-        <v>7.1</v>
+        <v>6.98</v>
       </c>
       <c r="Q12" s="397" t="n">
-        <v>6.74</v>
+        <v>6.49</v>
       </c>
       <c r="R12" s="397" t="n">
         <v>8.76</v>
@@ -13556,7 +13556,7 @@
         <v>7.67</v>
       </c>
       <c r="W12" s="397" t="n">
-        <v>3.29</v>
+        <v>3.44</v>
       </c>
       <c r="X12" s="397" t="n">
         <v>7.23</v>
@@ -13583,7 +13583,7 @@
         <v>10.28</v>
       </c>
       <c r="AF12" s="397" t="n">
-        <v>2.36</v>
+        <v>2.13</v>
       </c>
     </row>
     <row r="13" ht="12" customHeight="1" s="244">
@@ -13625,16 +13625,16 @@
         <v>1522.5</v>
       </c>
       <c r="N13" s="398" t="n">
-        <v>596.1</v>
+        <v>602.4</v>
       </c>
       <c r="O13" s="398" t="n">
         <v>1694</v>
       </c>
       <c r="P13" s="398" t="n">
-        <v>1460.2</v>
+        <v>1498</v>
       </c>
       <c r="Q13" s="398" t="n">
-        <v>1385</v>
+        <v>1392</v>
       </c>
       <c r="R13" s="398" t="n">
         <v>1850.8</v>
@@ -13652,7 +13652,7 @@
         <v>1533</v>
       </c>
       <c r="W13" s="398" t="n">
-        <v>561.1</v>
+        <v>611.4</v>
       </c>
       <c r="X13" s="398" t="n">
         <v>1370.6</v>
@@ -13679,7 +13679,7 @@
         <v>1998.8</v>
       </c>
       <c r="AF13" s="398" t="n">
-        <v>419.7</v>
+        <v>349</v>
       </c>
     </row>
     <row r="14" ht="12" customHeight="1" s="244">
@@ -15637,16 +15637,16 @@
         <v>6816</v>
       </c>
       <c r="N32" s="408" t="n">
-        <v>517</v>
+        <v>532</v>
       </c>
       <c r="O32" s="408" t="n">
         <v>9141</v>
       </c>
       <c r="P32" s="408" t="n">
-        <v>6076</v>
+        <v>6519</v>
       </c>
       <c r="Q32" s="408" t="n">
-        <v>5253</v>
+        <v>5327</v>
       </c>
       <c r="R32" s="408" t="n">
         <v>11661</v>
@@ -15664,7 +15664,7 @@
         <v>6946</v>
       </c>
       <c r="W32" s="408" t="n">
-        <v>278</v>
+        <v>555</v>
       </c>
       <c r="X32" s="408" t="n">
         <v>5105</v>
@@ -15691,7 +15691,7 @@
         <v>14409</v>
       </c>
       <c r="AF32" s="408" t="n">
-        <v>155</v>
+        <v>107</v>
       </c>
     </row>
     <row r="33" ht="12" customHeight="1" s="244">
@@ -16272,7 +16272,7 @@
       </c>
       <c r="E2" s="383" t="inlineStr">
         <is>
-          <t>TOPLAM ISI = 43868 W</t>
+          <t>TOPLAM ISI = 43738 W</t>
         </is>
       </c>
       <c r="F2" s="264" t="n"/>
@@ -17068,10 +17068,10 @@
         <v>7.87</v>
       </c>
       <c r="G12" s="397" t="n">
-        <v>7.21</v>
+        <v>6.98</v>
       </c>
       <c r="H12" s="397" t="n">
-        <v>7.94</v>
+        <v>6.49</v>
       </c>
       <c r="I12" s="397" t="n">
         <v>8.779999999999999</v>
@@ -17089,7 +17089,7 @@
         <v>7.66</v>
       </c>
       <c r="N12" s="397" t="n">
-        <v>3.28</v>
+        <v>3.44</v>
       </c>
       <c r="O12" s="397" t="n">
         <v>7.11</v>
@@ -17116,7 +17116,7 @@
         <v>10.3</v>
       </c>
       <c r="W12" s="397" t="n">
-        <v>2.36</v>
+        <v>2.13</v>
       </c>
       <c r="X12" s="397" t="n">
         <v>7.83</v>
@@ -17143,7 +17143,7 @@
         <v>7.61</v>
       </c>
       <c r="AF12" s="397" t="n">
-        <v>2.61</v>
+        <v>2.77</v>
       </c>
       <c r="AG12" s="426" t="n"/>
       <c r="AH12" s="426" t="n"/>
@@ -17181,10 +17181,10 @@
         <v>1695.4</v>
       </c>
       <c r="G13" s="398" t="n">
-        <v>1460.2</v>
+        <v>1498</v>
       </c>
       <c r="H13" s="398" t="n">
-        <v>1609.3</v>
+        <v>1392</v>
       </c>
       <c r="I13" s="398" t="n">
         <v>1850.8</v>
@@ -17202,7 +17202,7 @@
         <v>1533</v>
       </c>
       <c r="N13" s="398" t="n">
-        <v>560.7</v>
+        <v>582</v>
       </c>
       <c r="O13" s="398" t="n">
         <v>1341.2</v>
@@ -17229,7 +17229,7 @@
         <v>2005.1</v>
       </c>
       <c r="W13" s="398" t="n">
-        <v>419.7</v>
+        <v>349.3</v>
       </c>
       <c r="X13" s="398" t="n">
         <v>1688.4</v>
@@ -17256,7 +17256,7 @@
         <v>1522.5</v>
       </c>
       <c r="AF13" s="398" t="n">
-        <v>425.9</v>
+        <v>524.6</v>
       </c>
       <c r="AG13" s="428" t="n"/>
       <c r="AH13" s="428" t="n"/>
@@ -19509,10 +19509,10 @@
         <v>9162</v>
       </c>
       <c r="G32" s="408" t="n">
-        <v>6076</v>
+        <v>6519</v>
       </c>
       <c r="H32" s="408" t="n">
-        <v>7939</v>
+        <v>5327</v>
       </c>
       <c r="I32" s="408" t="n">
         <v>11661</v>
@@ -19530,7 +19530,7 @@
         <v>6946</v>
       </c>
       <c r="N32" s="408" t="n">
-        <v>277</v>
+        <v>299</v>
       </c>
       <c r="O32" s="408" t="n">
         <v>4810</v>
@@ -19557,7 +19557,7 @@
         <v>14535</v>
       </c>
       <c r="W32" s="408" t="n">
-        <v>155</v>
+        <v>108</v>
       </c>
       <c r="X32" s="408" t="n">
         <v>9058</v>
@@ -19584,7 +19584,7 @@
         <v>6816</v>
       </c>
       <c r="AF32" s="408" t="n">
-        <v>160</v>
+        <v>243</v>
       </c>
       <c r="AG32" s="434" t="n"/>
       <c r="AH32" s="434" t="n"/>
@@ -20022,7 +20022,7 @@
     <row r="38" ht="12.75" customHeight="1" s="244">
       <c r="B38" s="411" t="inlineStr">
         <is>
-          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): 101-1 (38.1 °C), 102-2 (37.1 °C), 102-3 (37.1 °C), 103-4 (37.8 °C), 104-5 (37.8 °C), 105-6 (37.7 °C), 105-7 (37.7 °C), 106-8 (32.0 °C) ...</t>
+          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): 101-1 (38.1 °C), 102-2 (38.1 °C), 102-3 (38.1 °C), 103-4 (37.8 °C), 104-5 (37.8 °C), 105-6 (37.7 °C), 105-7 (37.7 °C), 106-8 (32.0 °C) ...</t>
         </is>
       </c>
       <c r="F38" s="243" t="inlineStr">
@@ -20246,7 +20246,7 @@
       </c>
       <c r="E2" s="383" t="inlineStr">
         <is>
-          <t>TOPLAM ISI = 43759 W</t>
+          <t>TOPLAM ISI = 43519 W</t>
         </is>
       </c>
       <c r="F2" s="264" t="n"/>
@@ -21042,10 +21042,10 @@
         <v>7.57</v>
       </c>
       <c r="G12" s="397" t="n">
-        <v>7.19</v>
+        <v>6.98</v>
       </c>
       <c r="H12" s="397" t="n">
-        <v>7.96</v>
+        <v>6.46</v>
       </c>
       <c r="I12" s="397" t="n">
         <v>8.76</v>
@@ -21063,7 +21063,7 @@
         <v>7.64</v>
       </c>
       <c r="N12" s="397" t="n">
-        <v>3.33</v>
+        <v>3.49</v>
       </c>
       <c r="O12" s="397" t="n">
         <v>6.92</v>
@@ -21090,7 +21090,7 @@
         <v>10.51</v>
       </c>
       <c r="W12" s="397" t="n">
-        <v>2.33</v>
+        <v>2.11</v>
       </c>
       <c r="X12" s="397" t="n">
         <v>7.8</v>
@@ -21117,7 +21117,7 @@
         <v>8.07</v>
       </c>
       <c r="AF12" s="397" t="n">
-        <v>3.35</v>
+        <v>3.52</v>
       </c>
       <c r="AG12" s="426" t="n"/>
       <c r="AH12" s="426" t="n"/>
@@ -21155,10 +21155,10 @@
         <v>1597.8</v>
       </c>
       <c r="G13" s="398" t="n">
-        <v>1451.8</v>
+        <v>1488.9</v>
       </c>
       <c r="H13" s="398" t="n">
-        <v>1605.4</v>
+        <v>1378.3</v>
       </c>
       <c r="I13" s="398" t="n">
         <v>1848</v>
@@ -21176,7 +21176,7 @@
         <v>1526.3</v>
       </c>
       <c r="N13" s="398" t="n">
-        <v>621.2</v>
+        <v>627.5</v>
       </c>
       <c r="O13" s="398" t="n">
         <v>1288.4</v>
@@ -21203,7 +21203,7 @@
         <v>2005.9</v>
       </c>
       <c r="W13" s="398" t="n">
-        <v>420.3</v>
+        <v>344.1</v>
       </c>
       <c r="X13" s="398" t="n">
         <v>1679.7</v>
@@ -21230,7 +21230,7 @@
         <v>1545.2</v>
       </c>
       <c r="AF13" s="398" t="n">
-        <v>627.5</v>
+        <v>646.8</v>
       </c>
       <c r="AG13" s="428" t="n"/>
       <c r="AH13" s="428" t="n"/>
@@ -23483,10 +23483,10 @@
         <v>7783</v>
       </c>
       <c r="G32" s="408" t="n">
-        <v>5981</v>
+        <v>6410</v>
       </c>
       <c r="H32" s="408" t="n">
-        <v>7887</v>
+        <v>5184</v>
       </c>
       <c r="I32" s="408" t="n">
         <v>11613</v>
@@ -23504,7 +23504,7 @@
         <v>6864</v>
       </c>
       <c r="N32" s="408" t="n">
-        <v>579</v>
+        <v>596</v>
       </c>
       <c r="O32" s="408" t="n">
         <v>4306</v>
@@ -23531,7 +23531,7 @@
         <v>14549</v>
       </c>
       <c r="W32" s="408" t="n">
-        <v>156</v>
+        <v>104</v>
       </c>
       <c r="X32" s="408" t="n">
         <v>8930</v>
@@ -23558,7 +23558,7 @@
         <v>7100</v>
       </c>
       <c r="AF32" s="408" t="n">
-        <v>596</v>
+        <v>647</v>
       </c>
       <c r="AG32" s="434" t="n"/>
       <c r="AH32" s="434" t="n"/>
@@ -23996,7 +23996,7 @@
     <row r="38" ht="12.75" customHeight="1" s="244">
       <c r="B38" s="411" t="inlineStr">
         <is>
-          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): 201-1 (37.8 °C), 202-2 (37.1 °C), 202-3 (37.1 °C), 203-4 (37.8 °C), 204-5 (37.8 °C), 205-6 (37.7 °C), 205-7 (37.7 °C), 206-8 (31.9 °C) ...</t>
+          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): 201-1 (37.8 °C), 202-2 (38.0 °C), 202-3 (38.0 °C), 203-4 (37.8 °C), 204-5 (37.8 °C), 205-6 (37.7 °C), 205-7 (37.7 °C), 206-8 (31.9 °C) ...</t>
         </is>
       </c>
       <c r="F38" s="243" t="inlineStr">

</xml_diff>

<commit_message>
yerden2 tur 3: etiket sırası en büyük ölçeğe göre, TEKNİK RAPOR 1.4 negatif MODÜL notu (K-1), BENIOKU tur 3, kontrolör tur 3 PNG'leri ve kırpımlar
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RwXcqZmf9VPBpDgb8LPkn3
</commit_message>
<xml_diff>
--- a/proje/denemeler/yerden2/NB_YERDEN_ISITMA.xlsx
+++ b/proje/denemeler/yerden2/NB_YERDEN_ISITMA.xlsx
@@ -17,7 +17,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'kapak'!$A$1:$I$42</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'TEKNİK RAPOR'!$A$1:$H$40</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'TEKNİK RAPOR'!$A$1:$H$48</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'PETEK LİST'!$A$1:$P$76</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'YERDEN ISITMA'!$A$1:$N$76</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'MMO YERDEN ISITMA'!$A$1:$AF$47</definedName>
@@ -3829,7 +3829,7 @@
       <c r="A38" s="310" t="n"/>
       <c r="B38" s="313" t="inlineStr">
         <is>
-          <t>Boru PEX 16 x 2,0, boru aralığı 15 cm, duvardan kenar mesafesi 7,5 cm; devre boyu en çok 80 m.</t>
+          <t>Boru PEX 16 x 2,0, boru aralığı 15 cm, duvardan kenar mesafesi 7,5 cm (dar ıslak hacimlerde 5-6 cm); devre boyu en çok 80 m.</t>
         </is>
       </c>
       <c r="E38" s="243" t="n"/>
@@ -3858,8 +3858,16 @@
       <c r="H40" s="280" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1" s="244">
-      <c r="A41" s="310" t="n"/>
-      <c r="B41" s="313" t="n"/>
+      <c r="A41" s="310" t="inlineStr">
+        <is>
+          <t>1.4.</t>
+        </is>
+      </c>
+      <c r="B41" s="313" t="inlineStr">
+        <is>
+          <t>Not — "YERDEN ISITMA" (modülasyon) sayfasındaki negatif değerler:</t>
+        </is>
+      </c>
       <c r="E41" s="243" t="n"/>
       <c r="F41" s="317" t="n"/>
       <c r="G41" s="323" t="n"/>
@@ -3875,7 +3883,11 @@
     </row>
     <row r="43" ht="15" customHeight="1" s="244">
       <c r="A43" s="310" t="n"/>
-      <c r="B43" s="313" t="n"/>
+      <c r="B43" s="313" t="inlineStr">
+        <is>
+          <t>Sayfadaki G sütunu (MODÜL) şablon formülüdür: G = 76,263 − 0,539 × F, F = q = Q / A (W/m²). Şablon 17,5 W/m esası için kurulmuştur;</t>
+        </is>
+      </c>
       <c r="E43" s="243" t="n"/>
       <c r="F43" s="317" t="n"/>
       <c r="G43" s="323" t="n"/>
@@ -3883,7 +3895,11 @@
     </row>
     <row r="44" ht="15" customHeight="1" s="244">
       <c r="A44" s="310" t="n"/>
-      <c r="B44" s="313" t="n"/>
+      <c r="B44" s="313" t="inlineStr">
+        <is>
+          <t>q &gt; 141,5 W/m² olduğunda G negatif çıkar. Bu projede Q = 35 W/m × L ve boru yoğunluğu ≈ 6 m/m² olduğundan q ≈ 200-215 W/m² olur;</t>
+        </is>
+      </c>
       <c r="E44" s="243" t="n"/>
       <c r="F44" s="317" t="n"/>
       <c r="G44" s="323" t="n"/>
@@ -3891,7 +3907,11 @@
     </row>
     <row r="45" ht="15" customHeight="1" s="244">
       <c r="A45" s="310" t="n"/>
-      <c r="B45" s="313" t="n"/>
+      <c r="B45" s="313" t="inlineStr">
+        <is>
+          <t>bu yüzden G (MODÜL) ve H = D / G (m²) sütunlarında negatif değerler görünür. Bunlar bir ölçü değildir, yalnız formülün geçerlilik aralığı dışında olunduğunu gösterir.</t>
+        </is>
+      </c>
       <c r="E45" s="243" t="n"/>
       <c r="F45" s="317" t="n"/>
       <c r="G45" s="323" t="n"/>
@@ -3899,7 +3919,11 @@
     </row>
     <row r="46" ht="15" customHeight="1" s="244">
       <c r="A46" s="310" t="n"/>
-      <c r="B46" s="313" t="n"/>
+      <c r="B46" s="313" t="inlineStr">
+        <is>
+          <t>Formüller bozulmadan bırakılmıştır. Aynı esasla MMO sayfasında yüzey sıcaklığı ≈ 37,8 °C ve devre basınç kaybı Δpmax üstünde çıkar (sayfadaki uyarı satırları).</t>
+        </is>
+      </c>
       <c r="C46" s="324" t="n"/>
       <c r="D46" s="323" t="n"/>
       <c r="E46" s="243" t="n"/>
@@ -3909,7 +3933,11 @@
     </row>
     <row r="47" ht="15" customHeight="1" s="244">
       <c r="A47" s="310" t="n"/>
-      <c r="B47" s="313" t="n"/>
+      <c r="B47" s="313" t="inlineStr">
+        <is>
+          <t>Devre gücü esası (35 W/m × L, plan etiketleriyle aynı) proje sahibinin kararına bırakılmıştır; 17,5 W/m ya da ısı kaybı esasına geçilirse bu değerler olağan aralığa döner.</t>
+        </is>
+      </c>
       <c r="C47" s="324" t="n"/>
       <c r="D47" s="323" t="n"/>
       <c r="E47" s="243" t="n"/>

</xml_diff>

<commit_message>
yerden2 tur 4 (ara): wc+banyo serpantin klozet önü altından (kullanıcı gibi), klozet çentiği mahale katıldı, Ç.M. ön panel şeridi engel değil, ıslak hacimde kenar 2,5–3 ve 0,5 cm faz taraması
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RwXcqZmf9VPBpDgb8LPkn3
</commit_message>
<xml_diff>
--- a/proje/denemeler/yerden2/NB_YERDEN_ISITMA.xlsx
+++ b/proje/denemeler/yerden2/NB_YERDEN_ISITMA.xlsx
@@ -4680,7 +4680,7 @@
         </is>
       </c>
       <c r="D16" s="343" t="n">
-        <v>602.4</v>
+        <v>661.1</v>
       </c>
       <c r="E16" s="344" t="n">
         <v>35</v>
@@ -4690,7 +4690,7 @@
         <v/>
       </c>
       <c r="G16" s="340" t="n">
-        <v>17.21</v>
+        <v>18.89</v>
       </c>
       <c r="H16" s="340" t="n">
         <v>1</v>
@@ -4995,7 +4995,7 @@
         </is>
       </c>
       <c r="D23" s="343" t="n">
-        <v>611.4</v>
+        <v>671</v>
       </c>
       <c r="E23" s="344" t="n">
         <v>35</v>
@@ -5005,7 +5005,7 @@
         <v/>
       </c>
       <c r="G23" s="340" t="n">
-        <v>17.47</v>
+        <v>19.17</v>
       </c>
       <c r="H23" s="340" t="n">
         <v>1</v>
@@ -5310,7 +5310,7 @@
         </is>
       </c>
       <c r="D30" s="348" t="n">
-        <v>349</v>
+        <v>465.1</v>
       </c>
       <c r="E30" s="349" t="n">
         <v>35</v>
@@ -5320,7 +5320,7 @@
         <v/>
       </c>
       <c r="G30" s="345" t="n">
-        <v>9.970000000000001</v>
+        <v>13.29</v>
       </c>
       <c r="H30" s="345" t="n">
         <v>1</v>
@@ -5658,7 +5658,7 @@
         </is>
       </c>
       <c r="D38" s="348" t="n">
-        <v>582</v>
+        <v>670.2</v>
       </c>
       <c r="E38" s="349" t="n">
         <v>35</v>
@@ -5668,7 +5668,7 @@
         <v/>
       </c>
       <c r="G38" s="345" t="n">
-        <v>16.63</v>
+        <v>19.15</v>
       </c>
       <c r="H38" s="345" t="n">
         <v>1</v>
@@ -5973,7 +5973,7 @@
         </is>
       </c>
       <c r="D45" s="348" t="n">
-        <v>349.3</v>
+        <v>465.1</v>
       </c>
       <c r="E45" s="349" t="n">
         <v>35</v>
@@ -5983,7 +5983,7 @@
         <v/>
       </c>
       <c r="G45" s="345" t="n">
-        <v>9.98</v>
+        <v>13.29</v>
       </c>
       <c r="H45" s="345" t="n">
         <v>1</v>
@@ -6288,7 +6288,7 @@
         </is>
       </c>
       <c r="D52" s="348" t="n">
-        <v>524.6</v>
+        <v>560</v>
       </c>
       <c r="E52" s="349" t="n">
         <v>35</v>
@@ -6298,7 +6298,7 @@
         <v/>
       </c>
       <c r="G52" s="345" t="n">
-        <v>14.99</v>
+        <v>16</v>
       </c>
       <c r="H52" s="345" t="n">
         <v>1</v>
@@ -6636,7 +6636,7 @@
         </is>
       </c>
       <c r="D60" s="348" t="n">
-        <v>627.5</v>
+        <v>695.8</v>
       </c>
       <c r="E60" s="349" t="n">
         <v>35</v>
@@ -6646,7 +6646,7 @@
         <v/>
       </c>
       <c r="G60" s="345" t="n">
-        <v>17.93</v>
+        <v>19.88</v>
       </c>
       <c r="H60" s="345" t="n">
         <v>1</v>
@@ -6951,7 +6951,7 @@
         </is>
       </c>
       <c r="D67" s="348" t="n">
-        <v>344.1</v>
+        <v>460.2</v>
       </c>
       <c r="E67" s="349" t="n">
         <v>35</v>
@@ -6961,7 +6961,7 @@
         <v/>
       </c>
       <c r="G67" s="345" t="n">
-        <v>9.83</v>
+        <v>13.15</v>
       </c>
       <c r="H67" s="345" t="n">
         <v>1</v>
@@ -7266,7 +7266,7 @@
         </is>
       </c>
       <c r="D74" s="348" t="n">
-        <v>646.8</v>
+        <v>704.2</v>
       </c>
       <c r="E74" s="349" t="n">
         <v>35</v>
@@ -7276,7 +7276,7 @@
         <v/>
       </c>
       <c r="G74" s="345" t="n">
-        <v>18.48</v>
+        <v>20.12</v>
       </c>
       <c r="H74" s="345" t="n">
         <v>1</v>
@@ -12852,7 +12852,7 @@
       </c>
       <c r="E2" s="383" t="inlineStr">
         <is>
-          <t>TOPLAM ISI = 44002 W</t>
+          <t>TOPLAM ISI = 44237 W</t>
         </is>
       </c>
       <c r="F2" s="264" t="n"/>
@@ -13557,7 +13557,7 @@
         <v>7.61</v>
       </c>
       <c r="N12" s="397" t="n">
-        <v>3.39</v>
+        <v>3.54</v>
       </c>
       <c r="O12" s="397" t="n">
         <v>7.87</v>
@@ -13584,7 +13584,7 @@
         <v>7.67</v>
       </c>
       <c r="W12" s="397" t="n">
-        <v>3.44</v>
+        <v>3.6</v>
       </c>
       <c r="X12" s="397" t="n">
         <v>7.23</v>
@@ -13611,7 +13611,7 @@
         <v>10.28</v>
       </c>
       <c r="AF12" s="397" t="n">
-        <v>2.13</v>
+        <v>2.41</v>
       </c>
     </row>
     <row r="13" ht="12" customHeight="1" s="244">
@@ -13653,7 +13653,7 @@
         <v>1522.5</v>
       </c>
       <c r="N13" s="398" t="n">
-        <v>602.4</v>
+        <v>661.1</v>
       </c>
       <c r="O13" s="398" t="n">
         <v>1694</v>
@@ -13680,7 +13680,7 @@
         <v>1533</v>
       </c>
       <c r="W13" s="398" t="n">
-        <v>611.4</v>
+        <v>671</v>
       </c>
       <c r="X13" s="398" t="n">
         <v>1370.6</v>
@@ -13707,7 +13707,7 @@
         <v>1998.8</v>
       </c>
       <c r="AF13" s="398" t="n">
-        <v>349</v>
+        <v>465.1</v>
       </c>
     </row>
     <row r="14" ht="12" customHeight="1" s="244">
@@ -15665,7 +15665,7 @@
         <v>6816</v>
       </c>
       <c r="N32" s="408" t="n">
-        <v>532</v>
+        <v>688</v>
       </c>
       <c r="O32" s="408" t="n">
         <v>9141</v>
@@ -15692,7 +15692,7 @@
         <v>6946</v>
       </c>
       <c r="W32" s="408" t="n">
-        <v>555</v>
+        <v>716</v>
       </c>
       <c r="X32" s="408" t="n">
         <v>5105</v>
@@ -15719,7 +15719,7 @@
         <v>14409</v>
       </c>
       <c r="AF32" s="408" t="n">
-        <v>107</v>
+        <v>191</v>
       </c>
     </row>
     <row r="33" ht="12" customHeight="1" s="244">
@@ -16300,7 +16300,7 @@
       </c>
       <c r="E2" s="383" t="inlineStr">
         <is>
-          <t>TOPLAM ISI = 43738 W</t>
+          <t>TOPLAM ISI = 43977 W</t>
         </is>
       </c>
       <c r="F2" s="264" t="n"/>
@@ -17117,7 +17117,7 @@
         <v>7.66</v>
       </c>
       <c r="N12" s="397" t="n">
-        <v>3.44</v>
+        <v>3.59</v>
       </c>
       <c r="O12" s="397" t="n">
         <v>7.11</v>
@@ -17144,7 +17144,7 @@
         <v>10.3</v>
       </c>
       <c r="W12" s="397" t="n">
-        <v>2.13</v>
+        <v>2.41</v>
       </c>
       <c r="X12" s="397" t="n">
         <v>7.83</v>
@@ -17171,7 +17171,7 @@
         <v>7.61</v>
       </c>
       <c r="AF12" s="397" t="n">
-        <v>2.77</v>
+        <v>2.93</v>
       </c>
       <c r="AG12" s="426" t="n"/>
       <c r="AH12" s="426" t="n"/>
@@ -17230,7 +17230,7 @@
         <v>1533</v>
       </c>
       <c r="N13" s="398" t="n">
-        <v>582</v>
+        <v>670.2</v>
       </c>
       <c r="O13" s="398" t="n">
         <v>1341.2</v>
@@ -17257,7 +17257,7 @@
         <v>2005.1</v>
       </c>
       <c r="W13" s="398" t="n">
-        <v>349.3</v>
+        <v>465.1</v>
       </c>
       <c r="X13" s="398" t="n">
         <v>1688.4</v>
@@ -17284,7 +17284,7 @@
         <v>1522.5</v>
       </c>
       <c r="AF13" s="398" t="n">
-        <v>524.6</v>
+        <v>560</v>
       </c>
       <c r="AG13" s="428" t="n"/>
       <c r="AH13" s="428" t="n"/>
@@ -19558,7 +19558,7 @@
         <v>6946</v>
       </c>
       <c r="N32" s="408" t="n">
-        <v>299</v>
+        <v>714</v>
       </c>
       <c r="O32" s="408" t="n">
         <v>4810</v>
@@ -19585,7 +19585,7 @@
         <v>14535</v>
       </c>
       <c r="W32" s="408" t="n">
-        <v>108</v>
+        <v>191</v>
       </c>
       <c r="X32" s="408" t="n">
         <v>9058</v>
@@ -19612,7 +19612,7 @@
         <v>6816</v>
       </c>
       <c r="AF32" s="408" t="n">
-        <v>243</v>
+        <v>277</v>
       </c>
       <c r="AG32" s="434" t="n"/>
       <c r="AH32" s="434" t="n"/>
@@ -20274,7 +20274,7 @@
       </c>
       <c r="E2" s="383" t="inlineStr">
         <is>
-          <t>TOPLAM ISI = 43519 W</t>
+          <t>TOPLAM ISI = 43760 W</t>
         </is>
       </c>
       <c r="F2" s="264" t="n"/>
@@ -21091,7 +21091,7 @@
         <v>7.64</v>
       </c>
       <c r="N12" s="397" t="n">
-        <v>3.49</v>
+        <v>3.64</v>
       </c>
       <c r="O12" s="397" t="n">
         <v>6.92</v>
@@ -21118,7 +21118,7 @@
         <v>10.51</v>
       </c>
       <c r="W12" s="397" t="n">
-        <v>2.11</v>
+        <v>2.37</v>
       </c>
       <c r="X12" s="397" t="n">
         <v>7.8</v>
@@ -21145,7 +21145,7 @@
         <v>8.07</v>
       </c>
       <c r="AF12" s="397" t="n">
-        <v>3.52</v>
+        <v>3.67</v>
       </c>
       <c r="AG12" s="426" t="n"/>
       <c r="AH12" s="426" t="n"/>
@@ -21204,7 +21204,7 @@
         <v>1526.3</v>
       </c>
       <c r="N13" s="398" t="n">
-        <v>627.5</v>
+        <v>695.8</v>
       </c>
       <c r="O13" s="398" t="n">
         <v>1288.4</v>
@@ -21231,7 +21231,7 @@
         <v>2005.9</v>
       </c>
       <c r="W13" s="398" t="n">
-        <v>344.1</v>
+        <v>460.2</v>
       </c>
       <c r="X13" s="398" t="n">
         <v>1679.7</v>
@@ -21258,7 +21258,7 @@
         <v>1545.2</v>
       </c>
       <c r="AF13" s="398" t="n">
-        <v>646.8</v>
+        <v>704.2</v>
       </c>
       <c r="AG13" s="428" t="n"/>
       <c r="AH13" s="428" t="n"/>
@@ -23532,7 +23532,7 @@
         <v>6864</v>
       </c>
       <c r="N32" s="408" t="n">
-        <v>596</v>
+        <v>791</v>
       </c>
       <c r="O32" s="408" t="n">
         <v>4306</v>
@@ -23559,7 +23559,7 @@
         <v>14549</v>
       </c>
       <c r="W32" s="408" t="n">
-        <v>104</v>
+        <v>187</v>
       </c>
       <c r="X32" s="408" t="n">
         <v>8930</v>
@@ -23586,7 +23586,7 @@
         <v>7100</v>
       </c>
       <c r="AF32" s="408" t="n">
-        <v>647</v>
+        <v>818</v>
       </c>
       <c r="AG32" s="434" t="n"/>
       <c r="AH32" s="434" t="n"/>

</xml_diff>

<commit_message>
yerden2: tüm 81 devre kollektöre ayaklı (kesişme 0, aralık <4 cm 0, kapıdan geçiş, başka mahal 0); kombi hattı 8/9 daire; şema paneli kullanıcı bloğu görünümü; çıktılar yenilendi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RwXcqZmf9VPBpDgb8LPkn3
</commit_message>
<xml_diff>
--- a/proje/denemeler/yerden2/NB_YERDEN_ISITMA.xlsx
+++ b/proje/denemeler/yerden2/NB_YERDEN_ISITMA.xlsx
@@ -4410,7 +4410,7 @@
         </is>
       </c>
       <c r="D10" s="343" t="n">
-        <v>1688.4</v>
+        <v>1649.2</v>
       </c>
       <c r="E10" s="344" t="n">
         <v>35</v>
@@ -4420,7 +4420,7 @@
         <v/>
       </c>
       <c r="G10" s="340" t="n">
-        <v>48.24</v>
+        <v>47.12</v>
       </c>
       <c r="H10" s="340" t="n">
         <v>1</v>
@@ -4455,7 +4455,7 @@
         </is>
       </c>
       <c r="D11" s="343" t="n">
-        <v>2872.1</v>
+        <v>3369.8</v>
       </c>
       <c r="E11" s="344" t="n">
         <v>35</v>
@@ -4465,7 +4465,7 @@
         <v/>
       </c>
       <c r="G11" s="340" t="n">
-        <v>82.06</v>
+        <v>96.28</v>
       </c>
       <c r="H11" s="340" t="n">
         <v>2</v>
@@ -4500,7 +4500,7 @@
         </is>
       </c>
       <c r="D12" s="343" t="n">
-        <v>1850.8</v>
+        <v>2001</v>
       </c>
       <c r="E12" s="344" t="n">
         <v>35</v>
@@ -4510,7 +4510,7 @@
         <v/>
       </c>
       <c r="G12" s="340" t="n">
-        <v>52.88</v>
+        <v>57.17</v>
       </c>
       <c r="H12" s="340" t="n">
         <v>1</v>
@@ -4545,7 +4545,7 @@
         </is>
       </c>
       <c r="D13" s="343" t="n">
-        <v>1866.2</v>
+        <v>2088.8</v>
       </c>
       <c r="E13" s="344" t="n">
         <v>35</v>
@@ -4555,7 +4555,7 @@
         <v/>
       </c>
       <c r="G13" s="340" t="n">
-        <v>53.32</v>
+        <v>59.68</v>
       </c>
       <c r="H13" s="340" t="n">
         <v>1</v>
@@ -4590,7 +4590,7 @@
         </is>
       </c>
       <c r="D14" s="343" t="n">
-        <v>4240.9</v>
+        <v>4620.7</v>
       </c>
       <c r="E14" s="344" t="n">
         <v>35</v>
@@ -4600,7 +4600,7 @@
         <v/>
       </c>
       <c r="G14" s="340" t="n">
-        <v>121.17</v>
+        <v>132.02</v>
       </c>
       <c r="H14" s="340" t="n">
         <v>2</v>
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="D15" s="343" t="n">
-        <v>1522.5</v>
+        <v>202.3</v>
       </c>
       <c r="E15" s="344" t="n">
         <v>35</v>
@@ -4645,7 +4645,7 @@
         <v/>
       </c>
       <c r="G15" s="340" t="n">
-        <v>43.5</v>
+        <v>5.78</v>
       </c>
       <c r="H15" s="340" t="n">
         <v>1</v>
@@ -4680,7 +4680,7 @@
         </is>
       </c>
       <c r="D16" s="343" t="n">
-        <v>661.1</v>
+        <v>854</v>
       </c>
       <c r="E16" s="344" t="n">
         <v>35</v>
@@ -4690,7 +4690,7 @@
         <v/>
       </c>
       <c r="G16" s="340" t="n">
-        <v>18.89</v>
+        <v>24.4</v>
       </c>
       <c r="H16" s="340" t="n">
         <v>1</v>
@@ -4725,7 +4725,7 @@
         </is>
       </c>
       <c r="D17" s="343" t="n">
-        <v>1694</v>
+        <v>1374.1</v>
       </c>
       <c r="E17" s="344" t="n">
         <v>35</v>
@@ -4735,7 +4735,7 @@
         <v/>
       </c>
       <c r="G17" s="340" t="n">
-        <v>48.4</v>
+        <v>39.26</v>
       </c>
       <c r="H17" s="340" t="n">
         <v>1</v>
@@ -4770,7 +4770,7 @@
         </is>
       </c>
       <c r="D18" s="343" t="n">
-        <v>2889.9</v>
+        <v>3396.8</v>
       </c>
       <c r="E18" s="344" t="n">
         <v>35</v>
@@ -4780,7 +4780,7 @@
         <v/>
       </c>
       <c r="G18" s="340" t="n">
-        <v>82.56999999999999</v>
+        <v>97.05</v>
       </c>
       <c r="H18" s="340" t="n">
         <v>2</v>
@@ -4815,7 +4815,7 @@
         </is>
       </c>
       <c r="D19" s="343" t="n">
-        <v>1850.8</v>
+        <v>2002.4</v>
       </c>
       <c r="E19" s="344" t="n">
         <v>35</v>
@@ -4825,7 +4825,7 @@
         <v/>
       </c>
       <c r="G19" s="340" t="n">
-        <v>52.88</v>
+        <v>57.21</v>
       </c>
       <c r="H19" s="340" t="n">
         <v>1</v>
@@ -4860,7 +4860,7 @@
         </is>
       </c>
       <c r="D20" s="343" t="n">
-        <v>1860.6</v>
+        <v>2072</v>
       </c>
       <c r="E20" s="344" t="n">
         <v>35</v>
@@ -4870,7 +4870,7 @@
         <v/>
       </c>
       <c r="G20" s="340" t="n">
-        <v>53.16</v>
+        <v>59.2</v>
       </c>
       <c r="H20" s="340" t="n">
         <v>1</v>
@@ -4905,7 +4905,7 @@
         </is>
       </c>
       <c r="D21" s="343" t="n">
-        <v>4253.6</v>
+        <v>4647.3</v>
       </c>
       <c r="E21" s="344" t="n">
         <v>35</v>
@@ -4915,7 +4915,7 @@
         <v/>
       </c>
       <c r="G21" s="340" t="n">
-        <v>121.53</v>
+        <v>132.78</v>
       </c>
       <c r="H21" s="340" t="n">
         <v>2</v>
@@ -4950,7 +4950,7 @@
         </is>
       </c>
       <c r="D22" s="343" t="n">
-        <v>1533</v>
+        <v>183.4</v>
       </c>
       <c r="E22" s="344" t="n">
         <v>35</v>
@@ -4960,7 +4960,7 @@
         <v/>
       </c>
       <c r="G22" s="340" t="n">
-        <v>43.8</v>
+        <v>5.24</v>
       </c>
       <c r="H22" s="340" t="n">
         <v>1</v>
@@ -4995,7 +4995,7 @@
         </is>
       </c>
       <c r="D23" s="343" t="n">
-        <v>671</v>
+        <v>872.9</v>
       </c>
       <c r="E23" s="344" t="n">
         <v>35</v>
@@ -5005,7 +5005,7 @@
         <v/>
       </c>
       <c r="G23" s="340" t="n">
-        <v>19.17</v>
+        <v>24.94</v>
       </c>
       <c r="H23" s="340" t="n">
         <v>1</v>
@@ -5040,7 +5040,7 @@
         </is>
       </c>
       <c r="D24" s="343" t="n">
-        <v>1370.6</v>
+        <v>1010.1</v>
       </c>
       <c r="E24" s="344" t="n">
         <v>35</v>
@@ -5050,7 +5050,7 @@
         <v/>
       </c>
       <c r="G24" s="340" t="n">
-        <v>39.16</v>
+        <v>28.86</v>
       </c>
       <c r="H24" s="340" t="n">
         <v>1</v>
@@ -5085,7 +5085,7 @@
         </is>
       </c>
       <c r="D25" s="348" t="n">
-        <v>3031.7</v>
+        <v>3711.4</v>
       </c>
       <c r="E25" s="349" t="n">
         <v>35</v>
@@ -5095,7 +5095,7 @@
         <v/>
       </c>
       <c r="G25" s="345" t="n">
-        <v>86.62</v>
+        <v>106.04</v>
       </c>
       <c r="H25" s="345" t="n">
         <v>2</v>
@@ -5130,7 +5130,7 @@
         </is>
       </c>
       <c r="D26" s="348" t="n">
-        <v>1859.2</v>
+        <v>2216.9</v>
       </c>
       <c r="E26" s="349" t="n">
         <v>35</v>
@@ -5140,7 +5140,7 @@
         <v/>
       </c>
       <c r="G26" s="345" t="n">
-        <v>53.12</v>
+        <v>63.34</v>
       </c>
       <c r="H26" s="345" t="n">
         <v>1</v>
@@ -5175,7 +5175,7 @@
         </is>
       </c>
       <c r="D27" s="348" t="n">
-        <v>4437.3</v>
+        <v>4299.1</v>
       </c>
       <c r="E27" s="349" t="n">
         <v>35</v>
@@ -5185,7 +5185,7 @@
         <v/>
       </c>
       <c r="G27" s="345" t="n">
-        <v>126.78</v>
+        <v>122.83</v>
       </c>
       <c r="H27" s="345" t="n">
         <v>2</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="D28" s="348" t="n">
-        <v>1619.1</v>
+        <v>2157.1</v>
       </c>
       <c r="E28" s="349" t="n">
         <v>35</v>
@@ -5230,7 +5230,7 @@
         <v/>
       </c>
       <c r="G28" s="345" t="n">
-        <v>46.26</v>
+        <v>61.63</v>
       </c>
       <c r="H28" s="345" t="n">
         <v>1</v>
@@ -5265,7 +5265,7 @@
         </is>
       </c>
       <c r="D29" s="348" t="n">
-        <v>1998.8</v>
+        <v>915.6</v>
       </c>
       <c r="E29" s="349" t="n">
         <v>35</v>
@@ -5275,7 +5275,7 @@
         <v/>
       </c>
       <c r="G29" s="345" t="n">
-        <v>57.11</v>
+        <v>26.16</v>
       </c>
       <c r="H29" s="345" t="n">
         <v>1</v>
@@ -5310,7 +5310,7 @@
         </is>
       </c>
       <c r="D30" s="348" t="n">
-        <v>465.1</v>
+        <v>798.7</v>
       </c>
       <c r="E30" s="349" t="n">
         <v>35</v>
@@ -5320,7 +5320,7 @@
         <v/>
       </c>
       <c r="G30" s="345" t="n">
-        <v>13.29</v>
+        <v>22.82</v>
       </c>
       <c r="H30" s="345" t="n">
         <v>1</v>
@@ -5388,7 +5388,7 @@
         </is>
       </c>
       <c r="D32" s="348" t="n">
-        <v>1695.4</v>
+        <v>1375.5</v>
       </c>
       <c r="E32" s="349" t="n">
         <v>35</v>
@@ -5398,7 +5398,7 @@
         <v/>
       </c>
       <c r="G32" s="345" t="n">
-        <v>48.44</v>
+        <v>39.3</v>
       </c>
       <c r="H32" s="345" t="n">
         <v>1</v>
@@ -5433,7 +5433,7 @@
         </is>
       </c>
       <c r="D33" s="348" t="n">
-        <v>2889.9</v>
+        <v>3396.8</v>
       </c>
       <c r="E33" s="349" t="n">
         <v>35</v>
@@ -5443,7 +5443,7 @@
         <v/>
       </c>
       <c r="G33" s="345" t="n">
-        <v>82.56999999999999</v>
+        <v>97.05</v>
       </c>
       <c r="H33" s="345" t="n">
         <v>2</v>
@@ -5478,7 +5478,7 @@
         </is>
       </c>
       <c r="D34" s="348" t="n">
-        <v>1850.8</v>
+        <v>2002.4</v>
       </c>
       <c r="E34" s="349" t="n">
         <v>35</v>
@@ -5488,7 +5488,7 @@
         <v/>
       </c>
       <c r="G34" s="345" t="n">
-        <v>52.88</v>
+        <v>57.21</v>
       </c>
       <c r="H34" s="345" t="n">
         <v>1</v>
@@ -5523,7 +5523,7 @@
         </is>
       </c>
       <c r="D35" s="348" t="n">
-        <v>1860.6</v>
+        <v>2072</v>
       </c>
       <c r="E35" s="349" t="n">
         <v>35</v>
@@ -5533,7 +5533,7 @@
         <v/>
       </c>
       <c r="G35" s="345" t="n">
-        <v>53.16</v>
+        <v>59.2</v>
       </c>
       <c r="H35" s="345" t="n">
         <v>1</v>
@@ -5568,7 +5568,7 @@
         </is>
       </c>
       <c r="D36" s="348" t="n">
-        <v>4235.7</v>
+        <v>4634</v>
       </c>
       <c r="E36" s="349" t="n">
         <v>35</v>
@@ -5578,7 +5578,7 @@
         <v/>
       </c>
       <c r="G36" s="345" t="n">
-        <v>121.02</v>
+        <v>132.4</v>
       </c>
       <c r="H36" s="345" t="n">
         <v>2</v>
@@ -5613,7 +5613,7 @@
         </is>
       </c>
       <c r="D37" s="348" t="n">
-        <v>1533</v>
+        <v>183.4</v>
       </c>
       <c r="E37" s="349" t="n">
         <v>35</v>
@@ -5623,7 +5623,7 @@
         <v/>
       </c>
       <c r="G37" s="345" t="n">
-        <v>43.8</v>
+        <v>5.24</v>
       </c>
       <c r="H37" s="345" t="n">
         <v>1</v>
@@ -5658,7 +5658,7 @@
         </is>
       </c>
       <c r="D38" s="348" t="n">
-        <v>670.2</v>
+        <v>872.2</v>
       </c>
       <c r="E38" s="349" t="n">
         <v>35</v>
@@ -5668,7 +5668,7 @@
         <v/>
       </c>
       <c r="G38" s="345" t="n">
-        <v>19.15</v>
+        <v>24.92</v>
       </c>
       <c r="H38" s="345" t="n">
         <v>1</v>
@@ -5703,7 +5703,7 @@
         </is>
       </c>
       <c r="D39" s="348" t="n">
-        <v>1341.2</v>
+        <v>1271.2</v>
       </c>
       <c r="E39" s="349" t="n">
         <v>35</v>
@@ -5713,7 +5713,7 @@
         <v/>
       </c>
       <c r="G39" s="345" t="n">
-        <v>38.32</v>
+        <v>36.32</v>
       </c>
       <c r="H39" s="345" t="n">
         <v>1</v>
@@ -5748,7 +5748,7 @@
         </is>
       </c>
       <c r="D40" s="348" t="n">
-        <v>3031.7</v>
+        <v>3266.2</v>
       </c>
       <c r="E40" s="349" t="n">
         <v>35</v>
@@ -5758,7 +5758,7 @@
         <v/>
       </c>
       <c r="G40" s="345" t="n">
-        <v>86.62</v>
+        <v>93.31999999999999</v>
       </c>
       <c r="H40" s="345" t="n">
         <v>2</v>
@@ -5793,7 +5793,7 @@
         </is>
       </c>
       <c r="D41" s="348" t="n">
-        <v>1859.2</v>
+        <v>1985.9</v>
       </c>
       <c r="E41" s="349" t="n">
         <v>35</v>
@@ -5803,7 +5803,7 @@
         <v/>
       </c>
       <c r="G41" s="345" t="n">
-        <v>53.12</v>
+        <v>56.74</v>
       </c>
       <c r="H41" s="345" t="n">
         <v>1</v>
@@ -5838,7 +5838,7 @@
         </is>
       </c>
       <c r="D42" s="348" t="n">
-        <v>4299.8</v>
+        <v>4719.4</v>
       </c>
       <c r="E42" s="349" t="n">
         <v>35</v>
@@ -5848,7 +5848,7 @@
         <v/>
       </c>
       <c r="G42" s="345" t="n">
-        <v>122.85</v>
+        <v>134.84</v>
       </c>
       <c r="H42" s="345" t="n">
         <v>2</v>
@@ -5883,7 +5883,7 @@
         </is>
       </c>
       <c r="D43" s="348" t="n">
-        <v>1614.9</v>
+        <v>1931.3</v>
       </c>
       <c r="E43" s="349" t="n">
         <v>35</v>
@@ -5893,7 +5893,7 @@
         <v/>
       </c>
       <c r="G43" s="345" t="n">
-        <v>46.14</v>
+        <v>55.18</v>
       </c>
       <c r="H43" s="345" t="n">
         <v>1</v>
@@ -5928,7 +5928,7 @@
         </is>
       </c>
       <c r="D44" s="348" t="n">
-        <v>2005.1</v>
+        <v>449.4</v>
       </c>
       <c r="E44" s="349" t="n">
         <v>35</v>
@@ -5938,7 +5938,7 @@
         <v/>
       </c>
       <c r="G44" s="345" t="n">
-        <v>57.29</v>
+        <v>12.84</v>
       </c>
       <c r="H44" s="345" t="n">
         <v>1</v>
@@ -5973,7 +5973,7 @@
         </is>
       </c>
       <c r="D45" s="348" t="n">
-        <v>465.1</v>
+        <v>539</v>
       </c>
       <c r="E45" s="349" t="n">
         <v>35</v>
@@ -5983,7 +5983,7 @@
         <v/>
       </c>
       <c r="G45" s="345" t="n">
-        <v>13.29</v>
+        <v>15.4</v>
       </c>
       <c r="H45" s="345" t="n">
         <v>1</v>
@@ -6018,7 +6018,7 @@
         </is>
       </c>
       <c r="D46" s="348" t="n">
-        <v>1688.4</v>
+        <v>1653</v>
       </c>
       <c r="E46" s="349" t="n">
         <v>35</v>
@@ -6028,7 +6028,7 @@
         <v/>
       </c>
       <c r="G46" s="345" t="n">
-        <v>48.24</v>
+        <v>47.23</v>
       </c>
       <c r="H46" s="345" t="n">
         <v>1</v>
@@ -6063,7 +6063,7 @@
         </is>
       </c>
       <c r="D47" s="348" t="n">
-        <v>2877.7</v>
+        <v>3375.4</v>
       </c>
       <c r="E47" s="349" t="n">
         <v>35</v>
@@ -6073,7 +6073,7 @@
         <v/>
       </c>
       <c r="G47" s="345" t="n">
-        <v>82.22</v>
+        <v>96.44</v>
       </c>
       <c r="H47" s="345" t="n">
         <v>2</v>
@@ -6108,7 +6108,7 @@
         </is>
       </c>
       <c r="D48" s="348" t="n">
-        <v>1856.4</v>
+        <v>2006.5</v>
       </c>
       <c r="E48" s="349" t="n">
         <v>35</v>
@@ -6118,7 +6118,7 @@
         <v/>
       </c>
       <c r="G48" s="345" t="n">
-        <v>53.04</v>
+        <v>57.33</v>
       </c>
       <c r="H48" s="345" t="n">
         <v>1</v>
@@ -6153,7 +6153,7 @@
         </is>
       </c>
       <c r="D49" s="348" t="n">
-        <v>1872.8</v>
+        <v>2095.4</v>
       </c>
       <c r="E49" s="349" t="n">
         <v>35</v>
@@ -6163,7 +6163,7 @@
         <v/>
       </c>
       <c r="G49" s="345" t="n">
-        <v>53.51</v>
+        <v>59.87</v>
       </c>
       <c r="H49" s="345" t="n">
         <v>1</v>
@@ -6198,7 +6198,7 @@
         </is>
       </c>
       <c r="D50" s="348" t="n">
-        <v>4246.6</v>
+        <v>4626.3</v>
       </c>
       <c r="E50" s="349" t="n">
         <v>35</v>
@@ -6208,7 +6208,7 @@
         <v/>
       </c>
       <c r="G50" s="345" t="n">
-        <v>121.33</v>
+        <v>132.18</v>
       </c>
       <c r="H50" s="345" t="n">
         <v>2</v>
@@ -6243,7 +6243,7 @@
         </is>
       </c>
       <c r="D51" s="348" t="n">
-        <v>1522.5</v>
+        <v>202.3</v>
       </c>
       <c r="E51" s="349" t="n">
         <v>35</v>
@@ -6253,7 +6253,7 @@
         <v/>
       </c>
       <c r="G51" s="345" t="n">
-        <v>43.5</v>
+        <v>5.78</v>
       </c>
       <c r="H51" s="345" t="n">
         <v>1</v>
@@ -6288,7 +6288,7 @@
         </is>
       </c>
       <c r="D52" s="348" t="n">
-        <v>560</v>
+        <v>690.9</v>
       </c>
       <c r="E52" s="349" t="n">
         <v>35</v>
@@ -6298,7 +6298,7 @@
         <v/>
       </c>
       <c r="G52" s="345" t="n">
-        <v>16</v>
+        <v>19.74</v>
       </c>
       <c r="H52" s="345" t="n">
         <v>1</v>
@@ -6366,7 +6366,7 @@
         </is>
       </c>
       <c r="D54" s="348" t="n">
-        <v>1597.8</v>
+        <v>1760.5</v>
       </c>
       <c r="E54" s="349" t="n">
         <v>35</v>
@@ -6376,7 +6376,7 @@
         <v/>
       </c>
       <c r="G54" s="345" t="n">
-        <v>45.65</v>
+        <v>50.3</v>
       </c>
       <c r="H54" s="345" t="n">
         <v>1</v>
@@ -6411,7 +6411,7 @@
         </is>
       </c>
       <c r="D55" s="348" t="n">
-        <v>2867.2</v>
+        <v>3383.5</v>
       </c>
       <c r="E55" s="349" t="n">
         <v>35</v>
@@ -6421,7 +6421,7 @@
         <v/>
       </c>
       <c r="G55" s="345" t="n">
-        <v>81.92</v>
+        <v>96.67</v>
       </c>
       <c r="H55" s="345" t="n">
         <v>2</v>
@@ -6456,7 +6456,7 @@
         </is>
       </c>
       <c r="D56" s="348" t="n">
-        <v>1848</v>
+        <v>1999.6</v>
       </c>
       <c r="E56" s="349" t="n">
         <v>35</v>
@@ -6466,7 +6466,7 @@
         <v/>
       </c>
       <c r="G56" s="345" t="n">
-        <v>52.8</v>
+        <v>57.13</v>
       </c>
       <c r="H56" s="345" t="n">
         <v>1</v>
@@ -6501,7 +6501,7 @@
         </is>
       </c>
       <c r="D57" s="348" t="n">
-        <v>1859.2</v>
+        <v>2075.8</v>
       </c>
       <c r="E57" s="349" t="n">
         <v>35</v>
@@ -6511,7 +6511,7 @@
         <v/>
       </c>
       <c r="G57" s="345" t="n">
-        <v>53.12</v>
+        <v>59.31</v>
       </c>
       <c r="H57" s="345" t="n">
         <v>1</v>
@@ -6546,7 +6546,7 @@
         </is>
       </c>
       <c r="D58" s="348" t="n">
-        <v>4213.3</v>
+        <v>4611.6</v>
       </c>
       <c r="E58" s="349" t="n">
         <v>35</v>
@@ -6556,7 +6556,7 @@
         <v/>
       </c>
       <c r="G58" s="345" t="n">
-        <v>120.38</v>
+        <v>131.76</v>
       </c>
       <c r="H58" s="345" t="n">
         <v>2</v>
@@ -6591,7 +6591,7 @@
         </is>
       </c>
       <c r="D59" s="348" t="n">
-        <v>1526.3</v>
+        <v>255.8</v>
       </c>
       <c r="E59" s="349" t="n">
         <v>35</v>
@@ -6601,7 +6601,7 @@
         <v/>
       </c>
       <c r="G59" s="345" t="n">
-        <v>43.61</v>
+        <v>7.31</v>
       </c>
       <c r="H59" s="345" t="n">
         <v>1</v>
@@ -6636,7 +6636,7 @@
         </is>
       </c>
       <c r="D60" s="348" t="n">
-        <v>695.8</v>
+        <v>897.8</v>
       </c>
       <c r="E60" s="349" t="n">
         <v>35</v>
@@ -6646,7 +6646,7 @@
         <v/>
       </c>
       <c r="G60" s="345" t="n">
-        <v>19.88</v>
+        <v>25.65</v>
       </c>
       <c r="H60" s="345" t="n">
         <v>1</v>
@@ -6681,7 +6681,7 @@
         </is>
       </c>
       <c r="D61" s="348" t="n">
-        <v>1288.4</v>
+        <v>1253</v>
       </c>
       <c r="E61" s="349" t="n">
         <v>35</v>
@@ -6691,7 +6691,7 @@
         <v/>
       </c>
       <c r="G61" s="345" t="n">
-        <v>36.81</v>
+        <v>35.8</v>
       </c>
       <c r="H61" s="345" t="n">
         <v>1</v>
@@ -6726,7 +6726,7 @@
         </is>
       </c>
       <c r="D62" s="348" t="n">
-        <v>2937.2</v>
+        <v>3260.9</v>
       </c>
       <c r="E62" s="349" t="n">
         <v>35</v>
@@ -6736,7 +6736,7 @@
         <v/>
       </c>
       <c r="G62" s="345" t="n">
-        <v>83.92</v>
+        <v>93.17</v>
       </c>
       <c r="H62" s="345" t="n">
         <v>2</v>
@@ -6771,7 +6771,7 @@
         </is>
       </c>
       <c r="D63" s="348" t="n">
-        <v>1859.2</v>
+        <v>1982.4</v>
       </c>
       <c r="E63" s="349" t="n">
         <v>35</v>
@@ -6781,7 +6781,7 @@
         <v/>
       </c>
       <c r="G63" s="345" t="n">
-        <v>53.12</v>
+        <v>56.64</v>
       </c>
       <c r="H63" s="345" t="n">
         <v>1</v>
@@ -6816,7 +6816,7 @@
         </is>
       </c>
       <c r="D64" s="348" t="n">
-        <v>4288.6</v>
+        <v>4714.5</v>
       </c>
       <c r="E64" s="349" t="n">
         <v>35</v>
@@ -6826,7 +6826,7 @@
         <v/>
       </c>
       <c r="G64" s="345" t="n">
-        <v>122.53</v>
+        <v>134.7</v>
       </c>
       <c r="H64" s="345" t="n">
         <v>2</v>
@@ -6861,7 +6861,7 @@
         </is>
       </c>
       <c r="D65" s="348" t="n">
-        <v>1610.7</v>
+        <v>1927.1</v>
       </c>
       <c r="E65" s="349" t="n">
         <v>35</v>
@@ -6871,7 +6871,7 @@
         <v/>
       </c>
       <c r="G65" s="345" t="n">
-        <v>46.02</v>
+        <v>55.06</v>
       </c>
       <c r="H65" s="345" t="n">
         <v>1</v>
@@ -6906,7 +6906,7 @@
         </is>
       </c>
       <c r="D66" s="348" t="n">
-        <v>2005.9</v>
+        <v>450.8</v>
       </c>
       <c r="E66" s="349" t="n">
         <v>35</v>
@@ -6916,7 +6916,7 @@
         <v/>
       </c>
       <c r="G66" s="345" t="n">
-        <v>57.31</v>
+        <v>12.88</v>
       </c>
       <c r="H66" s="345" t="n">
         <v>1</v>
@@ -6951,7 +6951,7 @@
         </is>
       </c>
       <c r="D67" s="348" t="n">
-        <v>460.2</v>
+        <v>528.9</v>
       </c>
       <c r="E67" s="349" t="n">
         <v>35</v>
@@ -6961,7 +6961,7 @@
         <v/>
       </c>
       <c r="G67" s="345" t="n">
-        <v>13.15</v>
+        <v>15.11</v>
       </c>
       <c r="H67" s="345" t="n">
         <v>1</v>
@@ -6996,7 +6996,7 @@
         </is>
       </c>
       <c r="D68" s="348" t="n">
-        <v>1679.7</v>
+        <v>1660</v>
       </c>
       <c r="E68" s="349" t="n">
         <v>35</v>
@@ -7006,7 +7006,7 @@
         <v/>
       </c>
       <c r="G68" s="345" t="n">
-        <v>47.99</v>
+        <v>47.43</v>
       </c>
       <c r="H68" s="345" t="n">
         <v>1</v>
@@ -7041,7 +7041,7 @@
         </is>
       </c>
       <c r="D69" s="348" t="n">
-        <v>2864.4</v>
+        <v>3370.1</v>
       </c>
       <c r="E69" s="349" t="n">
         <v>35</v>
@@ -7051,7 +7051,7 @@
         <v/>
       </c>
       <c r="G69" s="345" t="n">
-        <v>81.84</v>
+        <v>96.29000000000001</v>
       </c>
       <c r="H69" s="345" t="n">
         <v>2</v>
@@ -7086,7 +7086,7 @@
         </is>
       </c>
       <c r="D70" s="348" t="n">
-        <v>1848</v>
+        <v>2006.9</v>
       </c>
       <c r="E70" s="349" t="n">
         <v>35</v>
@@ -7096,7 +7096,7 @@
         <v/>
       </c>
       <c r="G70" s="345" t="n">
-        <v>52.8</v>
+        <v>57.34</v>
       </c>
       <c r="H70" s="345" t="n">
         <v>1</v>
@@ -7131,7 +7131,7 @@
         </is>
       </c>
       <c r="D71" s="348" t="n">
-        <v>1864.8</v>
+        <v>2088.8</v>
       </c>
       <c r="E71" s="349" t="n">
         <v>35</v>
@@ -7141,7 +7141,7 @@
         <v/>
       </c>
       <c r="G71" s="345" t="n">
-        <v>53.28</v>
+        <v>59.68</v>
       </c>
       <c r="H71" s="345" t="n">
         <v>1</v>
@@ -7176,7 +7176,7 @@
         </is>
       </c>
       <c r="D72" s="348" t="n">
-        <v>4196.5</v>
+        <v>4603.9</v>
       </c>
       <c r="E72" s="349" t="n">
         <v>35</v>
@@ -7186,7 +7186,7 @@
         <v/>
       </c>
       <c r="G72" s="345" t="n">
-        <v>119.9</v>
+        <v>131.54</v>
       </c>
       <c r="H72" s="345" t="n">
         <v>2</v>
@@ -7221,7 +7221,7 @@
         </is>
       </c>
       <c r="D73" s="348" t="n">
-        <v>1545.2</v>
+        <v>174.3</v>
       </c>
       <c r="E73" s="349" t="n">
         <v>35</v>
@@ -7231,7 +7231,7 @@
         <v/>
       </c>
       <c r="G73" s="345" t="n">
-        <v>44.15</v>
+        <v>4.98</v>
       </c>
       <c r="H73" s="345" t="n">
         <v>1</v>
@@ -7266,7 +7266,7 @@
         </is>
       </c>
       <c r="D74" s="348" t="n">
-        <v>704.2</v>
+        <v>904</v>
       </c>
       <c r="E74" s="349" t="n">
         <v>35</v>
@@ -7276,7 +7276,7 @@
         <v/>
       </c>
       <c r="G74" s="345" t="n">
-        <v>20.12</v>
+        <v>25.83</v>
       </c>
       <c r="H74" s="345" t="n">
         <v>1</v>
@@ -12852,7 +12852,7 @@
       </c>
       <c r="E2" s="383" t="inlineStr">
         <is>
-          <t>TOPLAM ISI = 44237 W</t>
+          <t>TOPLAM ISI = 44443 W</t>
         </is>
       </c>
       <c r="F2" s="264" t="n"/>
@@ -12883,7 +12883,7 @@
       </c>
       <c r="E3" s="383" t="inlineStr">
         <is>
-          <t>MAX. BASINÇ KAYBI = 22298 Pa</t>
+          <t>MAX. BASINÇ KAYBI = 23920 Pa</t>
         </is>
       </c>
       <c r="F3" s="250" t="n"/>
@@ -13533,85 +13533,85 @@
       <c r="D12" s="261" t="n"/>
       <c r="E12" s="259" t="n"/>
       <c r="F12" s="397" t="n">
-        <v>7.83</v>
+        <v>6.92</v>
       </c>
       <c r="G12" s="397" t="n">
-        <v>7.11</v>
+        <v>6.47</v>
       </c>
       <c r="H12" s="397" t="n">
-        <v>6.49</v>
+        <v>6.97</v>
       </c>
       <c r="I12" s="397" t="n">
-        <v>8.779999999999999</v>
+        <v>8.48</v>
       </c>
       <c r="J12" s="397" t="n">
         <v>8.84</v>
       </c>
       <c r="K12" s="397" t="n">
-        <v>9.81</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="L12" s="397" t="n">
-        <v>10.29</v>
+        <v>10.24</v>
       </c>
       <c r="M12" s="397" t="n">
-        <v>7.61</v>
+        <v>1.17</v>
       </c>
       <c r="N12" s="397" t="n">
         <v>3.54</v>
       </c>
       <c r="O12" s="397" t="n">
-        <v>7.87</v>
+        <v>5.75</v>
       </c>
       <c r="P12" s="397" t="n">
-        <v>6.98</v>
+        <v>6.37</v>
       </c>
       <c r="Q12" s="397" t="n">
-        <v>6.49</v>
+        <v>6.96</v>
       </c>
       <c r="R12" s="397" t="n">
-        <v>8.76</v>
+        <v>8.43</v>
       </c>
       <c r="S12" s="397" t="n">
         <v>8.83</v>
       </c>
       <c r="T12" s="397" t="n">
-        <v>9.880000000000001</v>
+        <v>9.92</v>
       </c>
       <c r="U12" s="397" t="n">
-        <v>10.29</v>
+        <v>10.25</v>
       </c>
       <c r="V12" s="397" t="n">
-        <v>7.67</v>
+        <v>1.12</v>
       </c>
       <c r="W12" s="397" t="n">
         <v>3.6</v>
       </c>
       <c r="X12" s="397" t="n">
-        <v>7.23</v>
+        <v>4.26</v>
       </c>
       <c r="Y12" s="397" t="n">
-        <v>7.24</v>
+        <v>6.8</v>
       </c>
       <c r="Z12" s="397" t="n">
-        <v>7.08</v>
+        <v>7.31</v>
       </c>
       <c r="AA12" s="397" t="n">
         <v>8.640000000000001</v>
       </c>
       <c r="AB12" s="397" t="n">
-        <v>10.87</v>
+        <v>10.14</v>
       </c>
       <c r="AC12" s="397" t="n">
-        <v>10.08</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="AD12" s="397" t="n">
         <v>7.31</v>
       </c>
       <c r="AE12" s="397" t="n">
-        <v>10.28</v>
+        <v>4.95</v>
       </c>
       <c r="AF12" s="397" t="n">
-        <v>2.41</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="13" ht="12" customHeight="1" s="244">
@@ -13629,85 +13629,85 @@
       </c>
       <c r="E13" s="259" t="n"/>
       <c r="F13" s="398" t="n">
-        <v>1688.4</v>
+        <v>1649.2</v>
       </c>
       <c r="G13" s="398" t="n">
-        <v>1501.2</v>
+        <v>1621.2</v>
       </c>
       <c r="H13" s="398" t="n">
-        <v>1371</v>
+        <v>1748.6</v>
       </c>
       <c r="I13" s="398" t="n">
-        <v>1850.8</v>
+        <v>2001</v>
       </c>
       <c r="J13" s="398" t="n">
-        <v>1866.2</v>
+        <v>2088.8</v>
       </c>
       <c r="K13" s="398" t="n">
-        <v>2069.9</v>
+        <v>2266.6</v>
       </c>
       <c r="L13" s="398" t="n">
-        <v>2171.1</v>
+        <v>2354.1</v>
       </c>
       <c r="M13" s="398" t="n">
-        <v>1522.5</v>
+        <v>202.3</v>
       </c>
       <c r="N13" s="398" t="n">
-        <v>661.1</v>
+        <v>854</v>
       </c>
       <c r="O13" s="398" t="n">
-        <v>1694</v>
+        <v>1374.1</v>
       </c>
       <c r="P13" s="398" t="n">
-        <v>1498</v>
+        <v>1622.6</v>
       </c>
       <c r="Q13" s="398" t="n">
-        <v>1392</v>
+        <v>1774.1</v>
       </c>
       <c r="R13" s="398" t="n">
-        <v>1850.8</v>
+        <v>2002.4</v>
       </c>
       <c r="S13" s="398" t="n">
-        <v>1860.6</v>
+        <v>2072</v>
       </c>
       <c r="T13" s="398" t="n">
-        <v>2082.5</v>
+        <v>2286.2</v>
       </c>
       <c r="U13" s="398" t="n">
-        <v>2171.1</v>
+        <v>2361.1</v>
       </c>
       <c r="V13" s="398" t="n">
-        <v>1533</v>
+        <v>183.4</v>
       </c>
       <c r="W13" s="398" t="n">
-        <v>671</v>
+        <v>872.9</v>
       </c>
       <c r="X13" s="398" t="n">
-        <v>1370.6</v>
+        <v>1010.1</v>
       </c>
       <c r="Y13" s="398" t="n">
-        <v>1533</v>
+        <v>1789.6</v>
       </c>
       <c r="Z13" s="398" t="n">
-        <v>1498.7</v>
+        <v>1921.8</v>
       </c>
       <c r="AA13" s="398" t="n">
-        <v>1859.2</v>
+        <v>2216.9</v>
       </c>
       <c r="AB13" s="398" t="n">
-        <v>2301.6</v>
+        <v>2303</v>
       </c>
       <c r="AC13" s="398" t="n">
-        <v>2135.7</v>
+        <v>1996</v>
       </c>
       <c r="AD13" s="398" t="n">
-        <v>1619.1</v>
+        <v>2157.1</v>
       </c>
       <c r="AE13" s="398" t="n">
-        <v>1998.8</v>
+        <v>915.6</v>
       </c>
       <c r="AF13" s="398" t="n">
-        <v>465.1</v>
+        <v>798.7</v>
       </c>
     </row>
     <row r="14" ht="12" customHeight="1" s="244">
@@ -15641,85 +15641,85 @@
       </c>
       <c r="E32" s="259" t="n"/>
       <c r="F32" s="408" t="n">
-        <v>9058</v>
+        <v>8492</v>
       </c>
       <c r="G32" s="408" t="n">
-        <v>6556</v>
+        <v>8101</v>
       </c>
       <c r="H32" s="408" t="n">
-        <v>5109</v>
+        <v>9975</v>
       </c>
       <c r="I32" s="408" t="n">
-        <v>11661</v>
+        <v>14451</v>
       </c>
       <c r="J32" s="408" t="n">
-        <v>11930</v>
+        <v>16264</v>
       </c>
       <c r="K32" s="408" t="n">
-        <v>15862</v>
+        <v>20360</v>
       </c>
       <c r="L32" s="408" t="n">
-        <v>18086</v>
+        <v>22595</v>
       </c>
       <c r="M32" s="408" t="n">
-        <v>6816</v>
+        <v>36</v>
       </c>
       <c r="N32" s="408" t="n">
-        <v>688</v>
+        <v>1390</v>
       </c>
       <c r="O32" s="408" t="n">
-        <v>9141</v>
+        <v>5141</v>
       </c>
       <c r="P32" s="408" t="n">
-        <v>6519</v>
+        <v>8120</v>
       </c>
       <c r="Q32" s="408" t="n">
-        <v>5327</v>
+        <v>10381</v>
       </c>
       <c r="R32" s="408" t="n">
-        <v>11661</v>
+        <v>14479</v>
       </c>
       <c r="S32" s="408" t="n">
-        <v>11832</v>
+        <v>15906</v>
       </c>
       <c r="T32" s="408" t="n">
-        <v>16129</v>
+        <v>20848</v>
       </c>
       <c r="U32" s="408" t="n">
-        <v>18086</v>
+        <v>22781</v>
       </c>
       <c r="V32" s="408" t="n">
-        <v>6946</v>
+        <v>30</v>
       </c>
       <c r="W32" s="408" t="n">
-        <v>716</v>
+        <v>1476</v>
       </c>
       <c r="X32" s="408" t="n">
-        <v>5105</v>
+        <v>2205</v>
       </c>
       <c r="Y32" s="408" t="n">
-        <v>6946</v>
+        <v>10630</v>
       </c>
       <c r="Z32" s="408" t="n">
-        <v>6527</v>
+        <v>12934</v>
       </c>
       <c r="AA32" s="408" t="n">
-        <v>11807</v>
+        <v>19156</v>
       </c>
       <c r="AB32" s="408" t="n">
-        <v>21236</v>
+        <v>21272</v>
       </c>
       <c r="AC32" s="408" t="n">
-        <v>17288</v>
+        <v>14354</v>
       </c>
       <c r="AD32" s="408" t="n">
-        <v>8072</v>
+        <v>17767</v>
       </c>
       <c r="AE32" s="408" t="n">
-        <v>14409</v>
+        <v>1683</v>
       </c>
       <c r="AF32" s="408" t="n">
-        <v>191</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="33" ht="12" customHeight="1" s="244">
@@ -16081,7 +16081,7 @@
     <row r="38" ht="12.75" customHeight="1" s="244">
       <c r="B38" s="411" t="inlineStr">
         <is>
-          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): Z01-1 (38.1 °C), Z02-2 (37.8 °C), Z02-3 (37.8 °C), Z03-4 (37.8 °C), Z04-5 (37.8 °C), Z05-6 (37.8 °C), Z05-7 (37.8 °C), Z06-8 (32.0 °C) ...</t>
+          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): Z01-1 (39.9 °C), Z02-2 (40.8 °C), Z02-3 (40.8 °C), Z03-4 (39.7 °C), Z04-5 (39.7 °C), Z05-6 (39.2 °C), Z05-7 (39.2 °C), Z06-8 (29.8 °C) ...</t>
         </is>
       </c>
       <c r="H38" s="243" t="n"/>
@@ -16300,7 +16300,7 @@
       </c>
       <c r="E2" s="383" t="inlineStr">
         <is>
-          <t>TOPLAM ISI = 43977 W</t>
+          <t>TOPLAM ISI = 43349 W</t>
         </is>
       </c>
       <c r="F2" s="264" t="n"/>
@@ -16339,7 +16339,7 @@
       </c>
       <c r="E3" s="383" t="inlineStr">
         <is>
-          <t>MAX. BASINÇ KAYBI = 19058 Pa</t>
+          <t>MAX. BASINÇ KAYBI = 27181 Pa</t>
         </is>
       </c>
       <c r="F3" s="250" t="n"/>
@@ -17093,85 +17093,85 @@
       <c r="D12" s="261" t="n"/>
       <c r="E12" s="259" t="n"/>
       <c r="F12" s="397" t="n">
-        <v>7.87</v>
+        <v>5.76</v>
       </c>
       <c r="G12" s="397" t="n">
-        <v>6.98</v>
+        <v>6.37</v>
       </c>
       <c r="H12" s="397" t="n">
-        <v>6.49</v>
+        <v>6.96</v>
       </c>
       <c r="I12" s="397" t="n">
-        <v>8.779999999999999</v>
+        <v>8.460000000000001</v>
       </c>
       <c r="J12" s="397" t="n">
         <v>8.83</v>
       </c>
       <c r="K12" s="397" t="n">
-        <v>9.83</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="L12" s="397" t="n">
-        <v>10.3</v>
+        <v>10.25</v>
       </c>
       <c r="M12" s="397" t="n">
-        <v>7.66</v>
+        <v>1.12</v>
       </c>
       <c r="N12" s="397" t="n">
         <v>3.59</v>
       </c>
       <c r="O12" s="397" t="n">
-        <v>7.11</v>
+        <v>5.54</v>
       </c>
       <c r="P12" s="397" t="n">
-        <v>7.24</v>
+        <v>6.78</v>
       </c>
       <c r="Q12" s="397" t="n">
-        <v>7.07</v>
+        <v>7.33</v>
       </c>
       <c r="R12" s="397" t="n">
         <v>8.640000000000001</v>
       </c>
       <c r="S12" s="397" t="n">
-        <v>10.38</v>
+        <v>9.85</v>
       </c>
       <c r="T12" s="397" t="n">
-        <v>10.55</v>
+        <v>10.84</v>
       </c>
       <c r="U12" s="397" t="n">
         <v>7.29</v>
       </c>
       <c r="V12" s="397" t="n">
-        <v>10.3</v>
+        <v>2.64</v>
       </c>
       <c r="W12" s="397" t="n">
-        <v>2.41</v>
+        <v>1.14</v>
       </c>
       <c r="X12" s="397" t="n">
-        <v>7.83</v>
+        <v>6.9</v>
       </c>
       <c r="Y12" s="397" t="n">
-        <v>7.12</v>
+        <v>6.49</v>
       </c>
       <c r="Z12" s="397" t="n">
-        <v>6.5</v>
+        <v>6.98</v>
       </c>
       <c r="AA12" s="397" t="n">
-        <v>8.800000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="AB12" s="397" t="n">
         <v>8.880000000000001</v>
       </c>
       <c r="AC12" s="397" t="n">
-        <v>9.83</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="AD12" s="397" t="n">
-        <v>10.31</v>
+        <v>10.26</v>
       </c>
       <c r="AE12" s="397" t="n">
-        <v>7.61</v>
+        <v>1.17</v>
       </c>
       <c r="AF12" s="397" t="n">
-        <v>2.93</v>
+        <v>2.58</v>
       </c>
       <c r="AG12" s="426" t="n"/>
       <c r="AH12" s="426" t="n"/>
@@ -17206,85 +17206,85 @@
       </c>
       <c r="E13" s="259" t="n"/>
       <c r="F13" s="398" t="n">
-        <v>1695.4</v>
+        <v>1375.5</v>
       </c>
       <c r="G13" s="398" t="n">
-        <v>1498</v>
+        <v>1622.6</v>
       </c>
       <c r="H13" s="398" t="n">
-        <v>1392</v>
+        <v>1774.1</v>
       </c>
       <c r="I13" s="398" t="n">
-        <v>1850.8</v>
+        <v>2002.4</v>
       </c>
       <c r="J13" s="398" t="n">
-        <v>1860.6</v>
+        <v>2072</v>
       </c>
       <c r="K13" s="398" t="n">
-        <v>2068.5</v>
+        <v>2274.6</v>
       </c>
       <c r="L13" s="398" t="n">
-        <v>2167.2</v>
+        <v>2359.3</v>
       </c>
       <c r="M13" s="398" t="n">
-        <v>1533</v>
+        <v>183.4</v>
       </c>
       <c r="N13" s="398" t="n">
-        <v>670.2</v>
+        <v>872.2</v>
       </c>
       <c r="O13" s="398" t="n">
-        <v>1341.2</v>
+        <v>1271.2</v>
       </c>
       <c r="P13" s="398" t="n">
-        <v>1533</v>
+        <v>1569</v>
       </c>
       <c r="Q13" s="398" t="n">
-        <v>1498.7</v>
+        <v>1697.2</v>
       </c>
       <c r="R13" s="398" t="n">
-        <v>1859.2</v>
+        <v>1985.9</v>
       </c>
       <c r="S13" s="398" t="n">
-        <v>2132.2</v>
+        <v>2246</v>
       </c>
       <c r="T13" s="398" t="n">
-        <v>2167.6</v>
+        <v>2473.5</v>
       </c>
       <c r="U13" s="398" t="n">
-        <v>1614.9</v>
+        <v>1931.3</v>
       </c>
       <c r="V13" s="398" t="n">
-        <v>2005.1</v>
+        <v>449.4</v>
       </c>
       <c r="W13" s="398" t="n">
-        <v>465.1</v>
+        <v>539</v>
       </c>
       <c r="X13" s="398" t="n">
-        <v>1688.4</v>
+        <v>1653</v>
       </c>
       <c r="Y13" s="398" t="n">
-        <v>1505.3</v>
+        <v>1625.4</v>
       </c>
       <c r="Z13" s="398" t="n">
-        <v>1372.4</v>
+        <v>1750</v>
       </c>
       <c r="AA13" s="398" t="n">
-        <v>1856.4</v>
+        <v>2006.5</v>
       </c>
       <c r="AB13" s="398" t="n">
-        <v>1872.8</v>
+        <v>2095.4</v>
       </c>
       <c r="AC13" s="398" t="n">
-        <v>2072.7</v>
+        <v>2269.4</v>
       </c>
       <c r="AD13" s="398" t="n">
-        <v>2173.8</v>
+        <v>2356.9</v>
       </c>
       <c r="AE13" s="398" t="n">
-        <v>1522.5</v>
+        <v>202.3</v>
       </c>
       <c r="AF13" s="398" t="n">
-        <v>560</v>
+        <v>690.9</v>
       </c>
       <c r="AG13" s="428" t="n"/>
       <c r="AH13" s="428" t="n"/>
@@ -19534,85 +19534,85 @@
       </c>
       <c r="E32" s="259" t="n"/>
       <c r="F32" s="408" t="n">
-        <v>9162</v>
+        <v>5155</v>
       </c>
       <c r="G32" s="408" t="n">
-        <v>6519</v>
+        <v>8120</v>
       </c>
       <c r="H32" s="408" t="n">
-        <v>5327</v>
+        <v>10381</v>
       </c>
       <c r="I32" s="408" t="n">
-        <v>11661</v>
+        <v>14479</v>
       </c>
       <c r="J32" s="408" t="n">
-        <v>11832</v>
+        <v>15906</v>
       </c>
       <c r="K32" s="408" t="n">
-        <v>15833</v>
+        <v>20560</v>
       </c>
       <c r="L32" s="408" t="n">
-        <v>17998</v>
+        <v>22734</v>
       </c>
       <c r="M32" s="408" t="n">
-        <v>6946</v>
+        <v>30</v>
       </c>
       <c r="N32" s="408" t="n">
-        <v>714</v>
+        <v>1473</v>
       </c>
       <c r="O32" s="408" t="n">
-        <v>4810</v>
+        <v>4150</v>
       </c>
       <c r="P32" s="408" t="n">
-        <v>6946</v>
+        <v>7405</v>
       </c>
       <c r="Q32" s="408" t="n">
-        <v>6527</v>
+        <v>9188</v>
       </c>
       <c r="R32" s="408" t="n">
-        <v>11807</v>
+        <v>14154</v>
       </c>
       <c r="S32" s="408" t="n">
-        <v>17210</v>
+        <v>19854</v>
       </c>
       <c r="T32" s="408" t="n">
-        <v>18006</v>
+        <v>25887</v>
       </c>
       <c r="U32" s="408" t="n">
-        <v>8015</v>
+        <v>13109</v>
       </c>
       <c r="V32" s="408" t="n">
-        <v>14535</v>
+        <v>178</v>
       </c>
       <c r="W32" s="408" t="n">
-        <v>191</v>
+        <v>256</v>
       </c>
       <c r="X32" s="408" t="n">
-        <v>9058</v>
+        <v>8546</v>
       </c>
       <c r="Y32" s="408" t="n">
-        <v>6607</v>
+        <v>8159</v>
       </c>
       <c r="Z32" s="408" t="n">
-        <v>5123</v>
+        <v>9997</v>
       </c>
       <c r="AA32" s="408" t="n">
-        <v>11758</v>
+        <v>14563</v>
       </c>
       <c r="AB32" s="408" t="n">
-        <v>12047</v>
+        <v>16406</v>
       </c>
       <c r="AC32" s="408" t="n">
-        <v>15921</v>
+        <v>20429</v>
       </c>
       <c r="AD32" s="408" t="n">
-        <v>18150</v>
+        <v>22669</v>
       </c>
       <c r="AE32" s="408" t="n">
-        <v>6816</v>
+        <v>36</v>
       </c>
       <c r="AF32" s="408" t="n">
-        <v>277</v>
+        <v>776</v>
       </c>
       <c r="AG32" s="434" t="n"/>
       <c r="AH32" s="434" t="n"/>
@@ -20050,7 +20050,7 @@
     <row r="38" ht="12.75" customHeight="1" s="244">
       <c r="B38" s="411" t="inlineStr">
         <is>
-          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): 101-1 (38.1 °C), 102-2 (38.1 °C), 102-3 (38.1 °C), 103-4 (37.8 °C), 104-5 (37.8 °C), 105-6 (37.7 °C), 105-7 (37.7 °C), 106-8 (32.0 °C) ...</t>
+          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): 101-1 (39.9 °C), 102-2 (41.1 °C), 102-3 (41.1 °C), 103-4 (39.8 °C), 104-5 (39.6 °C), 105-6 (39.3 °C), 105-7 (39.3 °C), 106-8 (29.1 °C) ...</t>
         </is>
       </c>
       <c r="F38" s="243" t="inlineStr">
@@ -20274,7 +20274,7 @@
       </c>
       <c r="E2" s="383" t="inlineStr">
         <is>
-          <t>TOPLAM ISI = 43760 W</t>
+          <t>TOPLAM ISI = 43910 W</t>
         </is>
       </c>
       <c r="F2" s="264" t="n"/>
@@ -20313,7 +20313,7 @@
       </c>
       <c r="E3" s="383" t="inlineStr">
         <is>
-          <t>MAX. BASINÇ KAYBI = 18806 Pa</t>
+          <t>MAX. BASINÇ KAYBI = 28470 Pa</t>
         </is>
       </c>
       <c r="F3" s="250" t="n"/>
@@ -21070,79 +21070,79 @@
         <v>7.57</v>
       </c>
       <c r="G12" s="397" t="n">
-        <v>6.98</v>
+        <v>6.35</v>
       </c>
       <c r="H12" s="397" t="n">
-        <v>6.46</v>
+        <v>6.95</v>
       </c>
       <c r="I12" s="397" t="n">
-        <v>8.76</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="J12" s="397" t="n">
         <v>8.83</v>
       </c>
       <c r="K12" s="397" t="n">
-        <v>9.75</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="L12" s="397" t="n">
-        <v>10.28</v>
+        <v>10.23</v>
       </c>
       <c r="M12" s="397" t="n">
-        <v>7.64</v>
+        <v>1.24</v>
       </c>
       <c r="N12" s="397" t="n">
         <v>3.64</v>
       </c>
       <c r="O12" s="397" t="n">
-        <v>6.92</v>
+        <v>5.7</v>
       </c>
       <c r="P12" s="397" t="n">
-        <v>7.03</v>
+        <v>6.78</v>
       </c>
       <c r="Q12" s="397" t="n">
-        <v>7.18</v>
+        <v>7.38</v>
       </c>
       <c r="R12" s="397" t="n">
         <v>8.66</v>
       </c>
       <c r="S12" s="397" t="n">
-        <v>10.32</v>
+        <v>11.08</v>
       </c>
       <c r="T12" s="397" t="n">
-        <v>10.5</v>
+        <v>9.68</v>
       </c>
       <c r="U12" s="397" t="n">
         <v>7.28</v>
       </c>
       <c r="V12" s="397" t="n">
-        <v>10.51</v>
+        <v>2.81</v>
       </c>
       <c r="W12" s="397" t="n">
-        <v>2.37</v>
+        <v>2.06</v>
       </c>
       <c r="X12" s="397" t="n">
-        <v>7.8</v>
+        <v>6.9</v>
       </c>
       <c r="Y12" s="397" t="n">
-        <v>7.1</v>
+        <v>6.47</v>
       </c>
       <c r="Z12" s="397" t="n">
-        <v>6.48</v>
+        <v>6.96</v>
       </c>
       <c r="AA12" s="397" t="n">
-        <v>8.77</v>
+        <v>8.51</v>
       </c>
       <c r="AB12" s="397" t="n">
         <v>8.85</v>
       </c>
       <c r="AC12" s="397" t="n">
-        <v>9.68</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="AD12" s="397" t="n">
-        <v>10.3</v>
+        <v>10.26</v>
       </c>
       <c r="AE12" s="397" t="n">
-        <v>8.07</v>
+        <v>1.1</v>
       </c>
       <c r="AF12" s="397" t="n">
         <v>3.67</v>
@@ -21180,85 +21180,85 @@
       </c>
       <c r="E13" s="259" t="n"/>
       <c r="F13" s="398" t="n">
-        <v>1597.8</v>
+        <v>1760.5</v>
       </c>
       <c r="G13" s="398" t="n">
-        <v>1488.9</v>
+        <v>1616</v>
       </c>
       <c r="H13" s="398" t="n">
-        <v>1378.3</v>
+        <v>1767.5</v>
       </c>
       <c r="I13" s="398" t="n">
-        <v>1848</v>
+        <v>1999.6</v>
       </c>
       <c r="J13" s="398" t="n">
-        <v>1859.2</v>
+        <v>2075.8</v>
       </c>
       <c r="K13" s="398" t="n">
-        <v>2050.3</v>
+        <v>2256.4</v>
       </c>
       <c r="L13" s="398" t="n">
-        <v>2163</v>
+        <v>2355.2</v>
       </c>
       <c r="M13" s="398" t="n">
-        <v>1526.3</v>
+        <v>255.8</v>
       </c>
       <c r="N13" s="398" t="n">
-        <v>695.8</v>
+        <v>897.8</v>
       </c>
       <c r="O13" s="398" t="n">
-        <v>1288.4</v>
+        <v>1253</v>
       </c>
       <c r="P13" s="398" t="n">
-        <v>1453.5</v>
+        <v>1561.7</v>
       </c>
       <c r="Q13" s="398" t="n">
-        <v>1483.7</v>
+        <v>1699.2</v>
       </c>
       <c r="R13" s="398" t="n">
-        <v>1859.2</v>
+        <v>1982.4</v>
       </c>
       <c r="S13" s="398" t="n">
-        <v>2125.2</v>
+        <v>2515.5</v>
       </c>
       <c r="T13" s="398" t="n">
-        <v>2163.3</v>
+        <v>2199</v>
       </c>
       <c r="U13" s="398" t="n">
-        <v>1610.7</v>
+        <v>1927.1</v>
       </c>
       <c r="V13" s="398" t="n">
-        <v>2005.9</v>
+        <v>450.8</v>
       </c>
       <c r="W13" s="398" t="n">
-        <v>460.2</v>
+        <v>528.9</v>
       </c>
       <c r="X13" s="398" t="n">
-        <v>1679.7</v>
+        <v>1660</v>
       </c>
       <c r="Y13" s="398" t="n">
-        <v>1498</v>
+        <v>1622.6</v>
       </c>
       <c r="Z13" s="398" t="n">
-        <v>1366.4</v>
+        <v>1747.5</v>
       </c>
       <c r="AA13" s="398" t="n">
-        <v>1848</v>
+        <v>2006.9</v>
       </c>
       <c r="AB13" s="398" t="n">
-        <v>1864.8</v>
+        <v>2088.8</v>
       </c>
       <c r="AC13" s="398" t="n">
-        <v>2033.5</v>
+        <v>2239.7</v>
       </c>
       <c r="AD13" s="398" t="n">
-        <v>2163</v>
+        <v>2364.2</v>
       </c>
       <c r="AE13" s="398" t="n">
-        <v>1545.2</v>
+        <v>174.3</v>
       </c>
       <c r="AF13" s="398" t="n">
-        <v>704.2</v>
+        <v>904</v>
       </c>
       <c r="AG13" s="428" t="n"/>
       <c r="AH13" s="428" t="n"/>
@@ -21954,7 +21954,7 @@
         <f>U10+(U14/8.92)^0.91</f>
         <v/>
       </c>
-      <c r="V19" s="401">
+      <c r="V19" s="400">
         <f>V10+(V14/8.92)^0.91</f>
         <v/>
       </c>
@@ -21990,7 +21990,7 @@
         <f>AD10+(AD14/8.92)^0.91</f>
         <v/>
       </c>
-      <c r="AE19" s="401">
+      <c r="AE19" s="400">
         <f>AE10+(AE14/8.92)^0.91</f>
         <v/>
       </c>
@@ -23508,85 +23508,85 @@
       </c>
       <c r="E32" s="259" t="n"/>
       <c r="F32" s="408" t="n">
-        <v>7783</v>
+        <v>10162</v>
       </c>
       <c r="G32" s="408" t="n">
-        <v>6410</v>
+        <v>8029</v>
       </c>
       <c r="H32" s="408" t="n">
-        <v>5184</v>
+        <v>10274</v>
       </c>
       <c r="I32" s="408" t="n">
-        <v>11613</v>
+        <v>14423</v>
       </c>
       <c r="J32" s="408" t="n">
-        <v>11807</v>
+        <v>15988</v>
       </c>
       <c r="K32" s="408" t="n">
-        <v>15452</v>
+        <v>20110</v>
       </c>
       <c r="L32" s="408" t="n">
-        <v>17902</v>
+        <v>22623</v>
       </c>
       <c r="M32" s="408" t="n">
-        <v>6864</v>
+        <v>58</v>
       </c>
       <c r="N32" s="408" t="n">
-        <v>791</v>
+        <v>1595</v>
       </c>
       <c r="O32" s="408" t="n">
-        <v>4306</v>
+        <v>3989</v>
       </c>
       <c r="P32" s="408" t="n">
-        <v>6000</v>
+        <v>7310</v>
       </c>
       <c r="Q32" s="408" t="n">
-        <v>6348</v>
+        <v>9219</v>
       </c>
       <c r="R32" s="408" t="n">
-        <v>11807</v>
+        <v>14086</v>
       </c>
       <c r="S32" s="408" t="n">
-        <v>17055</v>
+        <v>27114</v>
       </c>
       <c r="T32" s="408" t="n">
-        <v>17910</v>
+        <v>18735</v>
       </c>
       <c r="U32" s="408" t="n">
-        <v>7958</v>
+        <v>13031</v>
       </c>
       <c r="V32" s="408" t="n">
-        <v>14549</v>
+        <v>179</v>
       </c>
       <c r="W32" s="408" t="n">
-        <v>187</v>
+        <v>247</v>
       </c>
       <c r="X32" s="408" t="n">
-        <v>8930</v>
+        <v>8646</v>
       </c>
       <c r="Y32" s="408" t="n">
-        <v>6519</v>
+        <v>8120</v>
       </c>
       <c r="Z32" s="408" t="n">
-        <v>5062</v>
+        <v>9958</v>
       </c>
       <c r="AA32" s="408" t="n">
-        <v>11613</v>
+        <v>14570</v>
       </c>
       <c r="AB32" s="408" t="n">
-        <v>11905</v>
+        <v>16264</v>
       </c>
       <c r="AC32" s="408" t="n">
-        <v>15107</v>
+        <v>19701</v>
       </c>
       <c r="AD32" s="408" t="n">
-        <v>17902</v>
+        <v>22864</v>
       </c>
       <c r="AE32" s="408" t="n">
-        <v>7100</v>
+        <v>27</v>
       </c>
       <c r="AF32" s="408" t="n">
-        <v>818</v>
+        <v>1626</v>
       </c>
       <c r="AG32" s="434" t="n"/>
       <c r="AH32" s="434" t="n"/>
@@ -24024,7 +24024,7 @@
     <row r="38" ht="12.75" customHeight="1" s="244">
       <c r="B38" s="411" t="inlineStr">
         <is>
-          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): 201-1 (37.8 °C), 202-2 (38.0 °C), 202-3 (38.0 °C), 203-4 (37.8 °C), 204-5 (37.8 °C), 205-6 (37.7 °C), 205-7 (37.7 °C), 206-8 (31.9 °C) ...</t>
+          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (25 devre): 201-1 (39.4 °C), 202-2 (41.1 °C), 202-3 (41.1 °C), 203-4 (39.8 °C), 204-5 (39.6 °C), 205-6 (39.3 °C), 205-7 (39.3 °C), 206-8 (32.4 °C) ...</t>
         </is>
       </c>
       <c r="F38" s="243" t="inlineStr">

</xml_diff>

<commit_message>
yerden2: hol devre etiketi değer sütununa göre kendi serpantininde; tur 5 çıktıları, kontrolör raporu, kırpımlar
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RwXcqZmf9VPBpDgb8LPkn3
</commit_message>
<xml_diff>
--- a/proje/denemeler/yerden2/NB_YERDEN_ISITMA.xlsx
+++ b/proje/denemeler/yerden2/NB_YERDEN_ISITMA.xlsx
@@ -4500,7 +4500,7 @@
         </is>
       </c>
       <c r="D12" s="343" t="n">
-        <v>2001</v>
+        <v>2084.2</v>
       </c>
       <c r="E12" s="344" t="n">
         <v>35</v>
@@ -4510,7 +4510,7 @@
         <v/>
       </c>
       <c r="G12" s="340" t="n">
-        <v>57.17</v>
+        <v>59.55</v>
       </c>
       <c r="H12" s="340" t="n">
         <v>1</v>
@@ -4815,7 +4815,7 @@
         </is>
       </c>
       <c r="D19" s="343" t="n">
-        <v>2002.4</v>
+        <v>2090.5</v>
       </c>
       <c r="E19" s="344" t="n">
         <v>35</v>
@@ -4825,7 +4825,7 @@
         <v/>
       </c>
       <c r="G19" s="340" t="n">
-        <v>57.21</v>
+        <v>59.73</v>
       </c>
       <c r="H19" s="340" t="n">
         <v>1</v>
@@ -5175,7 +5175,7 @@
         </is>
       </c>
       <c r="D27" s="348" t="n">
-        <v>4299.1</v>
+        <v>4301.5</v>
       </c>
       <c r="E27" s="349" t="n">
         <v>35</v>
@@ -5185,7 +5185,7 @@
         <v/>
       </c>
       <c r="G27" s="345" t="n">
-        <v>122.83</v>
+        <v>122.9</v>
       </c>
       <c r="H27" s="345" t="n">
         <v>2</v>
@@ -5265,7 +5265,7 @@
         </is>
       </c>
       <c r="D29" s="348" t="n">
-        <v>915.6</v>
+        <v>869.8</v>
       </c>
       <c r="E29" s="349" t="n">
         <v>35</v>
@@ -5275,7 +5275,7 @@
         <v/>
       </c>
       <c r="G29" s="345" t="n">
-        <v>26.16</v>
+        <v>24.85</v>
       </c>
       <c r="H29" s="345" t="n">
         <v>1</v>
@@ -5310,7 +5310,7 @@
         </is>
       </c>
       <c r="D30" s="348" t="n">
-        <v>798.7</v>
+        <v>1053.8</v>
       </c>
       <c r="E30" s="349" t="n">
         <v>35</v>
@@ -5320,7 +5320,7 @@
         <v/>
       </c>
       <c r="G30" s="345" t="n">
-        <v>22.82</v>
+        <v>30.11</v>
       </c>
       <c r="H30" s="345" t="n">
         <v>1</v>
@@ -5478,7 +5478,7 @@
         </is>
       </c>
       <c r="D34" s="348" t="n">
-        <v>2002.4</v>
+        <v>2090.5</v>
       </c>
       <c r="E34" s="349" t="n">
         <v>35</v>
@@ -5488,7 +5488,7 @@
         <v/>
       </c>
       <c r="G34" s="345" t="n">
-        <v>57.21</v>
+        <v>59.73</v>
       </c>
       <c r="H34" s="345" t="n">
         <v>1</v>
@@ -5703,7 +5703,7 @@
         </is>
       </c>
       <c r="D39" s="348" t="n">
-        <v>1271.2</v>
+        <v>1285.2</v>
       </c>
       <c r="E39" s="349" t="n">
         <v>35</v>
@@ -5713,7 +5713,7 @@
         <v/>
       </c>
       <c r="G39" s="345" t="n">
-        <v>36.32</v>
+        <v>36.72</v>
       </c>
       <c r="H39" s="345" t="n">
         <v>1</v>
@@ -5838,7 +5838,7 @@
         </is>
       </c>
       <c r="D42" s="348" t="n">
-        <v>4719.4</v>
+        <v>4733.4</v>
       </c>
       <c r="E42" s="349" t="n">
         <v>35</v>
@@ -5848,7 +5848,7 @@
         <v/>
       </c>
       <c r="G42" s="345" t="n">
-        <v>134.84</v>
+        <v>135.24</v>
       </c>
       <c r="H42" s="345" t="n">
         <v>2</v>
@@ -5928,7 +5928,7 @@
         </is>
       </c>
       <c r="D44" s="348" t="n">
-        <v>449.4</v>
+        <v>641.5</v>
       </c>
       <c r="E44" s="349" t="n">
         <v>35</v>
@@ -5938,7 +5938,7 @@
         <v/>
       </c>
       <c r="G44" s="345" t="n">
-        <v>12.84</v>
+        <v>18.33</v>
       </c>
       <c r="H44" s="345" t="n">
         <v>1</v>
@@ -5973,7 +5973,7 @@
         </is>
       </c>
       <c r="D45" s="348" t="n">
-        <v>539</v>
+        <v>791.7</v>
       </c>
       <c r="E45" s="349" t="n">
         <v>35</v>
@@ -5983,7 +5983,7 @@
         <v/>
       </c>
       <c r="G45" s="345" t="n">
-        <v>15.4</v>
+        <v>22.62</v>
       </c>
       <c r="H45" s="345" t="n">
         <v>1</v>
@@ -6108,7 +6108,7 @@
         </is>
       </c>
       <c r="D48" s="348" t="n">
-        <v>2006.5</v>
+        <v>2089.8</v>
       </c>
       <c r="E48" s="349" t="n">
         <v>35</v>
@@ -6118,7 +6118,7 @@
         <v/>
       </c>
       <c r="G48" s="345" t="n">
-        <v>57.33</v>
+        <v>59.71</v>
       </c>
       <c r="H48" s="345" t="n">
         <v>1</v>
@@ -6288,7 +6288,7 @@
         </is>
       </c>
       <c r="D52" s="348" t="n">
-        <v>690.9</v>
+        <v>731.1</v>
       </c>
       <c r="E52" s="349" t="n">
         <v>35</v>
@@ -6298,7 +6298,7 @@
         <v/>
       </c>
       <c r="G52" s="345" t="n">
-        <v>19.74</v>
+        <v>20.89</v>
       </c>
       <c r="H52" s="345" t="n">
         <v>1</v>
@@ -6456,7 +6456,7 @@
         </is>
       </c>
       <c r="D56" s="348" t="n">
-        <v>1999.6</v>
+        <v>2087.8</v>
       </c>
       <c r="E56" s="349" t="n">
         <v>35</v>
@@ -6466,7 +6466,7 @@
         <v/>
       </c>
       <c r="G56" s="345" t="n">
-        <v>57.13</v>
+        <v>59.65</v>
       </c>
       <c r="H56" s="345" t="n">
         <v>1</v>
@@ -6951,7 +6951,7 @@
         </is>
       </c>
       <c r="D67" s="348" t="n">
-        <v>528.9</v>
+        <v>786.4</v>
       </c>
       <c r="E67" s="349" t="n">
         <v>35</v>
@@ -6961,7 +6961,7 @@
         <v/>
       </c>
       <c r="G67" s="345" t="n">
-        <v>15.11</v>
+        <v>22.47</v>
       </c>
       <c r="H67" s="345" t="n">
         <v>1</v>
@@ -7086,7 +7086,7 @@
         </is>
       </c>
       <c r="D70" s="348" t="n">
-        <v>2006.9</v>
+        <v>2094.8</v>
       </c>
       <c r="E70" s="349" t="n">
         <v>35</v>
@@ -7096,7 +7096,7 @@
         <v/>
       </c>
       <c r="G70" s="345" t="n">
-        <v>57.34</v>
+        <v>59.85</v>
       </c>
       <c r="H70" s="345" t="n">
         <v>1</v>
@@ -12852,7 +12852,7 @@
       </c>
       <c r="E2" s="383" t="inlineStr">
         <is>
-          <t>TOPLAM ISI = 44443 W</t>
+          <t>TOPLAM ISI = 44827 W</t>
         </is>
       </c>
       <c r="F2" s="264" t="n"/>
@@ -13542,7 +13542,7 @@
         <v>6.97</v>
       </c>
       <c r="I12" s="397" t="n">
-        <v>8.48</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="J12" s="397" t="n">
         <v>8.84</v>
@@ -13569,7 +13569,7 @@
         <v>6.96</v>
       </c>
       <c r="R12" s="397" t="n">
-        <v>8.43</v>
+        <v>8.76</v>
       </c>
       <c r="S12" s="397" t="n">
         <v>8.83</v>
@@ -13590,28 +13590,28 @@
         <v>4.26</v>
       </c>
       <c r="Y12" s="397" t="n">
-        <v>6.8</v>
+        <v>6.82</v>
       </c>
       <c r="Z12" s="397" t="n">
-        <v>7.31</v>
+        <v>7.33</v>
       </c>
       <c r="AA12" s="397" t="n">
         <v>8.640000000000001</v>
       </c>
       <c r="AB12" s="397" t="n">
-        <v>10.14</v>
+        <v>11.14</v>
       </c>
       <c r="AC12" s="397" t="n">
-        <v>8.789999999999999</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="AD12" s="397" t="n">
         <v>7.31</v>
       </c>
       <c r="AE12" s="397" t="n">
-        <v>4.95</v>
+        <v>4.9</v>
       </c>
       <c r="AF12" s="397" t="n">
-        <v>1.12</v>
+        <v>2.41</v>
       </c>
     </row>
     <row r="13" ht="12" customHeight="1" s="244">
@@ -13638,7 +13638,7 @@
         <v>1748.6</v>
       </c>
       <c r="I13" s="398" t="n">
-        <v>2001</v>
+        <v>2084.2</v>
       </c>
       <c r="J13" s="398" t="n">
         <v>2088.8</v>
@@ -13665,7 +13665,7 @@
         <v>1774.1</v>
       </c>
       <c r="R13" s="398" t="n">
-        <v>2002.4</v>
+        <v>2090.5</v>
       </c>
       <c r="S13" s="398" t="n">
         <v>2072</v>
@@ -13695,19 +13695,19 @@
         <v>2216.9</v>
       </c>
       <c r="AB13" s="398" t="n">
-        <v>2303</v>
+        <v>2306.8</v>
       </c>
       <c r="AC13" s="398" t="n">
-        <v>1996</v>
+        <v>1994.7</v>
       </c>
       <c r="AD13" s="398" t="n">
         <v>2157.1</v>
       </c>
       <c r="AE13" s="398" t="n">
-        <v>915.6</v>
+        <v>869.8</v>
       </c>
       <c r="AF13" s="398" t="n">
-        <v>798.7</v>
+        <v>1053.8</v>
       </c>
     </row>
     <row r="14" ht="12" customHeight="1" s="244">
@@ -15650,7 +15650,7 @@
         <v>9975</v>
       </c>
       <c r="I32" s="408" t="n">
-        <v>14451</v>
+        <v>16166</v>
       </c>
       <c r="J32" s="408" t="n">
         <v>16264</v>
@@ -15677,7 +15677,7 @@
         <v>10381</v>
       </c>
       <c r="R32" s="408" t="n">
-        <v>14479</v>
+        <v>16301</v>
       </c>
       <c r="S32" s="408" t="n">
         <v>15906</v>
@@ -15707,19 +15707,19 @@
         <v>19156</v>
       </c>
       <c r="AB32" s="408" t="n">
-        <v>21272</v>
+        <v>21370</v>
       </c>
       <c r="AC32" s="408" t="n">
-        <v>14354</v>
+        <v>14326</v>
       </c>
       <c r="AD32" s="408" t="n">
         <v>17767</v>
       </c>
       <c r="AE32" s="408" t="n">
-        <v>1683</v>
+        <v>1462</v>
       </c>
       <c r="AF32" s="408" t="n">
-        <v>1156</v>
+        <v>2478</v>
       </c>
     </row>
     <row r="33" ht="12" customHeight="1" s="244">
@@ -16081,7 +16081,7 @@
     <row r="38" ht="12.75" customHeight="1" s="244">
       <c r="B38" s="411" t="inlineStr">
         <is>
-          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): Z01-1 (39.9 °C), Z02-2 (40.8 °C), Z02-3 (40.8 °C), Z03-4 (39.7 °C), Z04-5 (39.7 °C), Z05-6 (39.2 °C), Z05-7 (39.2 °C), Z06-8 (29.8 °C) ...</t>
+          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): Z01-1 (39.9 °C), Z02-2 (40.8 °C), Z02-3 (40.8 °C), Z03-4 (39.8 °C), Z04-5 (39.7 °C), Z05-6 (39.2 °C), Z05-7 (39.2 °C), Z06-8 (29.8 °C) ...</t>
         </is>
       </c>
       <c r="H38" s="243" t="n"/>
@@ -16300,7 +16300,7 @@
       </c>
       <c r="E2" s="383" t="inlineStr">
         <is>
-          <t>TOPLAM ISI = 43349 W</t>
+          <t>TOPLAM ISI = 44033 W</t>
         </is>
       </c>
       <c r="F2" s="264" t="n"/>
@@ -16339,7 +16339,7 @@
       </c>
       <c r="E3" s="383" t="inlineStr">
         <is>
-          <t>MAX. BASINÇ KAYBI = 27181 Pa</t>
+          <t>MAX. BASINÇ KAYBI = 27393 Pa</t>
         </is>
       </c>
       <c r="F3" s="250" t="n"/>
@@ -17102,7 +17102,7 @@
         <v>6.96</v>
       </c>
       <c r="I12" s="397" t="n">
-        <v>8.460000000000001</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="J12" s="397" t="n">
         <v>8.83</v>
@@ -17123,28 +17123,28 @@
         <v>5.54</v>
       </c>
       <c r="P12" s="397" t="n">
-        <v>6.78</v>
+        <v>6.79</v>
       </c>
       <c r="Q12" s="397" t="n">
-        <v>7.33</v>
+        <v>7.35</v>
       </c>
       <c r="R12" s="397" t="n">
         <v>8.640000000000001</v>
       </c>
       <c r="S12" s="397" t="n">
-        <v>9.85</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="T12" s="397" t="n">
-        <v>10.84</v>
+        <v>10.87</v>
       </c>
       <c r="U12" s="397" t="n">
         <v>7.29</v>
       </c>
       <c r="V12" s="397" t="n">
-        <v>2.64</v>
+        <v>2.07</v>
       </c>
       <c r="W12" s="397" t="n">
-        <v>1.14</v>
+        <v>2.41</v>
       </c>
       <c r="X12" s="397" t="n">
         <v>6.9</v>
@@ -17156,7 +17156,7 @@
         <v>6.98</v>
       </c>
       <c r="AA12" s="397" t="n">
-        <v>8.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="AB12" s="397" t="n">
         <v>8.880000000000001</v>
@@ -17171,7 +17171,7 @@
         <v>1.17</v>
       </c>
       <c r="AF12" s="397" t="n">
-        <v>2.58</v>
+        <v>2.93</v>
       </c>
       <c r="AG12" s="426" t="n"/>
       <c r="AH12" s="426" t="n"/>
@@ -17215,7 +17215,7 @@
         <v>1774.1</v>
       </c>
       <c r="I13" s="398" t="n">
-        <v>2002.4</v>
+        <v>2090.5</v>
       </c>
       <c r="J13" s="398" t="n">
         <v>2072</v>
@@ -17233,7 +17233,7 @@
         <v>872.2</v>
       </c>
       <c r="O13" s="398" t="n">
-        <v>1271.2</v>
+        <v>1285.2</v>
       </c>
       <c r="P13" s="398" t="n">
         <v>1569</v>
@@ -17245,19 +17245,19 @@
         <v>1985.9</v>
       </c>
       <c r="S13" s="398" t="n">
-        <v>2246</v>
+        <v>2253</v>
       </c>
       <c r="T13" s="398" t="n">
-        <v>2473.5</v>
+        <v>2480.5</v>
       </c>
       <c r="U13" s="398" t="n">
         <v>1931.3</v>
       </c>
       <c r="V13" s="398" t="n">
-        <v>449.4</v>
+        <v>641.5</v>
       </c>
       <c r="W13" s="398" t="n">
-        <v>539</v>
+        <v>791.7</v>
       </c>
       <c r="X13" s="398" t="n">
         <v>1653</v>
@@ -17269,7 +17269,7 @@
         <v>1750</v>
       </c>
       <c r="AA13" s="398" t="n">
-        <v>2006.5</v>
+        <v>2089.8</v>
       </c>
       <c r="AB13" s="398" t="n">
         <v>2095.4</v>
@@ -17284,7 +17284,7 @@
         <v>202.3</v>
       </c>
       <c r="AF13" s="398" t="n">
-        <v>690.9</v>
+        <v>731.1</v>
       </c>
       <c r="AG13" s="428" t="n"/>
       <c r="AH13" s="428" t="n"/>
@@ -19543,7 +19543,7 @@
         <v>10381</v>
       </c>
       <c r="I32" s="408" t="n">
-        <v>14479</v>
+        <v>16301</v>
       </c>
       <c r="J32" s="408" t="n">
         <v>15906</v>
@@ -19561,7 +19561,7 @@
         <v>1473</v>
       </c>
       <c r="O32" s="408" t="n">
-        <v>4150</v>
+        <v>4277</v>
       </c>
       <c r="P32" s="408" t="n">
         <v>7405</v>
@@ -19573,19 +19573,19 @@
         <v>14154</v>
       </c>
       <c r="S32" s="408" t="n">
-        <v>19854</v>
+        <v>20025</v>
       </c>
       <c r="T32" s="408" t="n">
-        <v>25887</v>
+        <v>26089</v>
       </c>
       <c r="U32" s="408" t="n">
         <v>13109</v>
       </c>
       <c r="V32" s="408" t="n">
-        <v>178</v>
+        <v>633</v>
       </c>
       <c r="W32" s="408" t="n">
-        <v>256</v>
+        <v>1129</v>
       </c>
       <c r="X32" s="408" t="n">
         <v>8546</v>
@@ -19597,7 +19597,7 @@
         <v>9997</v>
       </c>
       <c r="AA32" s="408" t="n">
-        <v>14563</v>
+        <v>16286</v>
       </c>
       <c r="AB32" s="408" t="n">
         <v>16406</v>
@@ -19612,7 +19612,7 @@
         <v>36</v>
       </c>
       <c r="AF32" s="408" t="n">
-        <v>776</v>
+        <v>907</v>
       </c>
       <c r="AG32" s="434" t="n"/>
       <c r="AH32" s="434" t="n"/>
@@ -20050,7 +20050,7 @@
     <row r="38" ht="12.75" customHeight="1" s="244">
       <c r="B38" s="411" t="inlineStr">
         <is>
-          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): 101-1 (39.9 °C), 102-2 (41.1 °C), 102-3 (41.1 °C), 103-4 (39.8 °C), 104-5 (39.6 °C), 105-6 (39.3 °C), 105-7 (39.3 °C), 106-8 (29.1 °C) ...</t>
+          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): 101-1 (39.9 °C), 102-2 (41.1 °C), 102-3 (41.1 °C), 103-4 (39.9 °C), 104-5 (39.6 °C), 105-6 (39.3 °C), 105-7 (39.3 °C), 106-8 (29.1 °C) ...</t>
         </is>
       </c>
       <c r="F38" s="243" t="inlineStr">
@@ -20274,7 +20274,7 @@
       </c>
       <c r="E2" s="383" t="inlineStr">
         <is>
-          <t>TOPLAM ISI = 43910 W</t>
+          <t>TOPLAM ISI = 44344 W</t>
         </is>
       </c>
       <c r="F2" s="264" t="n"/>
@@ -21076,7 +21076,7 @@
         <v>6.95</v>
       </c>
       <c r="I12" s="397" t="n">
-        <v>8.449999999999999</v>
+        <v>8.76</v>
       </c>
       <c r="J12" s="397" t="n">
         <v>8.83</v>
@@ -21118,7 +21118,7 @@
         <v>2.81</v>
       </c>
       <c r="W12" s="397" t="n">
-        <v>2.06</v>
+        <v>2.37</v>
       </c>
       <c r="X12" s="397" t="n">
         <v>6.9</v>
@@ -21130,7 +21130,7 @@
         <v>6.96</v>
       </c>
       <c r="AA12" s="397" t="n">
-        <v>8.51</v>
+        <v>8.77</v>
       </c>
       <c r="AB12" s="397" t="n">
         <v>8.85</v>
@@ -21189,7 +21189,7 @@
         <v>1767.5</v>
       </c>
       <c r="I13" s="398" t="n">
-        <v>1999.6</v>
+        <v>2087.8</v>
       </c>
       <c r="J13" s="398" t="n">
         <v>2075.8</v>
@@ -21231,7 +21231,7 @@
         <v>450.8</v>
       </c>
       <c r="W13" s="398" t="n">
-        <v>528.9</v>
+        <v>786.4</v>
       </c>
       <c r="X13" s="398" t="n">
         <v>1660</v>
@@ -21243,7 +21243,7 @@
         <v>1747.5</v>
       </c>
       <c r="AA13" s="398" t="n">
-        <v>2006.9</v>
+        <v>2094.8</v>
       </c>
       <c r="AB13" s="398" t="n">
         <v>2088.8</v>
@@ -23517,7 +23517,7 @@
         <v>10274</v>
       </c>
       <c r="I32" s="408" t="n">
-        <v>14423</v>
+        <v>16241</v>
       </c>
       <c r="J32" s="408" t="n">
         <v>15988</v>
@@ -23559,7 +23559,7 @@
         <v>179</v>
       </c>
       <c r="W32" s="408" t="n">
-        <v>247</v>
+        <v>1108</v>
       </c>
       <c r="X32" s="408" t="n">
         <v>8646</v>
@@ -23571,7 +23571,7 @@
         <v>9958</v>
       </c>
       <c r="AA32" s="408" t="n">
-        <v>14570</v>
+        <v>16391</v>
       </c>
       <c r="AB32" s="408" t="n">
         <v>16264</v>
@@ -24024,7 +24024,7 @@
     <row r="38" ht="12.75" customHeight="1" s="244">
       <c r="B38" s="411" t="inlineStr">
         <is>
-          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (25 devre): 201-1 (39.4 °C), 202-2 (41.1 °C), 202-3 (41.1 °C), 203-4 (39.8 °C), 204-5 (39.6 °C), 205-6 (39.3 °C), 205-7 (39.3 °C), 206-8 (32.4 °C) ...</t>
+          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (25 devre): 201-1 (39.4 °C), 202-2 (41.1 °C), 202-3 (41.1 °C), 203-4 (39.9 °C), 204-5 (39.6 °C), 205-6 (39.3 °C), 205-7 (39.3 °C), 206-8 (32.4 °C) ...</t>
         </is>
       </c>
       <c r="F38" s="243" t="inlineStr">

</xml_diff>

<commit_message>
WIP (durdurulan iş, onaysız): sihhi2/yerden2 yarım değişiklikler
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RwXcqZmf9VPBpDgb8LPkn3
</commit_message>
<xml_diff>
--- a/proje/denemeler/yerden2/NB_YERDEN_ISITMA.xlsx
+++ b/proje/denemeler/yerden2/NB_YERDEN_ISITMA.xlsx
@@ -12983,40 +12983,40 @@
       <c r="D7" s="389" t="n"/>
       <c r="E7" s="391" t="n"/>
       <c r="F7" s="392" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G7" s="392" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H7" s="392" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I7" s="392" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J7" s="392" t="n">
         <v>5</v>
       </c>
       <c r="K7" s="392" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L7" s="392" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="M7" s="392" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="N7" s="392" t="n">
         <v>9</v>
       </c>
       <c r="O7" s="392" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="P7" s="392" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q7" s="392" t="n">
         <v>11</v>
-      </c>
-      <c r="Q7" s="392" t="n">
-        <v>12</v>
       </c>
       <c r="R7" s="392" t="n">
         <v>13</v>
@@ -13031,37 +13031,37 @@
         <v>16</v>
       </c>
       <c r="V7" s="392" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="W7" s="392" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="X7" s="392" t="n">
         <v>19</v>
       </c>
       <c r="Y7" s="392" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="Z7" s="392" t="n">
         <v>21</v>
       </c>
       <c r="AA7" s="392" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="AB7" s="392" t="n">
+        <v>26</v>
+      </c>
+      <c r="AC7" s="392" t="n">
+        <v>27</v>
+      </c>
+      <c r="AD7" s="392" t="n">
         <v>23</v>
       </c>
-      <c r="AC7" s="392" t="n">
+      <c r="AE7" s="392" t="n">
+        <v>25</v>
+      </c>
+      <c r="AF7" s="392" t="n">
         <v>24</v>
-      </c>
-      <c r="AD7" s="392" t="n">
-        <v>25</v>
-      </c>
-      <c r="AE7" s="392" t="n">
-        <v>26</v>
-      </c>
-      <c r="AF7" s="392" t="n">
-        <v>27</v>
       </c>
     </row>
     <row r="8" ht="12" customHeight="1" s="244">
@@ -16081,7 +16081,7 @@
     <row r="38" ht="12.75" customHeight="1" s="244">
       <c r="B38" s="411" t="inlineStr">
         <is>
-          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): Z01-1 (39.9 °C), Z02-2 (40.8 °C), Z02-3 (40.8 °C), Z03-4 (39.8 °C), Z04-5 (39.7 °C), Z05-6 (39.2 °C), Z05-7 (39.2 °C), Z06-8 (29.8 °C) ...</t>
+          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): Z01-2 (39.9 °C), Z02-7 (40.8 °C), Z02-8 (40.8 °C), Z03-6 (39.8 °C), Z04-5 (39.7 °C), Z05-4 (39.2 °C), Z05-3 (39.2 °C), Z06-1 (29.8 °C) ...</t>
         </is>
       </c>
       <c r="H38" s="243" t="n"/>
@@ -16458,13 +16458,13 @@
       <c r="D7" s="389" t="n"/>
       <c r="E7" s="391" t="n"/>
       <c r="F7" s="392" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G7" s="392" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" s="392" t="n">
         <v>2</v>
-      </c>
-      <c r="H7" s="392" t="n">
-        <v>3</v>
       </c>
       <c r="I7" s="392" t="n">
         <v>4</v>
@@ -16479,61 +16479,61 @@
         <v>7</v>
       </c>
       <c r="M7" s="392" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N7" s="392" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="O7" s="392" t="n">
+        <v>18</v>
+      </c>
+      <c r="P7" s="392" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q7" s="392" t="n">
+        <v>11</v>
+      </c>
+      <c r="R7" s="392" t="n">
         <v>10</v>
       </c>
-      <c r="P7" s="392" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q7" s="392" t="n">
-        <v>12</v>
-      </c>
-      <c r="R7" s="392" t="n">
+      <c r="S7" s="392" t="n">
+        <v>15</v>
+      </c>
+      <c r="T7" s="392" t="n">
+        <v>16</v>
+      </c>
+      <c r="U7" s="392" t="n">
         <v>13</v>
-      </c>
-      <c r="S7" s="392" t="n">
-        <v>14</v>
-      </c>
-      <c r="T7" s="392" t="n">
-        <v>15</v>
-      </c>
-      <c r="U7" s="392" t="n">
-        <v>16</v>
       </c>
       <c r="V7" s="392" t="n">
         <v>17</v>
       </c>
       <c r="W7" s="392" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="X7" s="392" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Y7" s="392" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="Z7" s="392" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="AA7" s="392" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="AB7" s="392" t="n">
         <v>23</v>
       </c>
       <c r="AC7" s="392" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="AD7" s="392" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="AE7" s="392" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="AF7" s="392" t="n">
         <v>27</v>
@@ -20050,7 +20050,7 @@
     <row r="38" ht="12.75" customHeight="1" s="244">
       <c r="B38" s="411" t="inlineStr">
         <is>
-          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): 101-1 (39.9 °C), 102-2 (41.1 °C), 102-3 (41.1 °C), 103-4 (39.9 °C), 104-5 (39.6 °C), 105-6 (39.3 °C), 105-7 (39.3 °C), 106-8 (29.1 °C) ...</t>
+          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): 101-8 (39.9 °C), 102-3 (41.1 °C), 102-2 (41.1 °C), 103-4 (39.9 °C), 104-5 (39.6 °C), 105-6 (39.3 °C), 105-7 (39.3 °C), 106-9 (29.1 °C) ...</t>
         </is>
       </c>
       <c r="F38" s="243" t="inlineStr">
@@ -20432,13 +20432,13 @@
       <c r="D7" s="389" t="n"/>
       <c r="E7" s="391" t="n"/>
       <c r="F7" s="392" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G7" s="392" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" s="392" t="n">
         <v>2</v>
-      </c>
-      <c r="H7" s="392" t="n">
-        <v>3</v>
       </c>
       <c r="I7" s="392" t="n">
         <v>4</v>
@@ -20453,61 +20453,61 @@
         <v>7</v>
       </c>
       <c r="M7" s="392" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N7" s="392" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="O7" s="392" t="n">
+        <v>18</v>
+      </c>
+      <c r="P7" s="392" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q7" s="392" t="n">
+        <v>11</v>
+      </c>
+      <c r="R7" s="392" t="n">
         <v>10</v>
       </c>
-      <c r="P7" s="392" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q7" s="392" t="n">
-        <v>12</v>
-      </c>
-      <c r="R7" s="392" t="n">
+      <c r="S7" s="392" t="n">
+        <v>16</v>
+      </c>
+      <c r="T7" s="392" t="n">
+        <v>17</v>
+      </c>
+      <c r="U7" s="392" t="n">
         <v>13</v>
       </c>
-      <c r="S7" s="392" t="n">
+      <c r="V7" s="392" t="n">
+        <v>15</v>
+      </c>
+      <c r="W7" s="392" t="n">
         <v>14</v>
       </c>
-      <c r="T7" s="392" t="n">
-        <v>15</v>
-      </c>
-      <c r="U7" s="392" t="n">
-        <v>16</v>
-      </c>
-      <c r="V7" s="392" t="n">
-        <v>17</v>
-      </c>
-      <c r="W7" s="392" t="n">
-        <v>18</v>
-      </c>
       <c r="X7" s="392" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Y7" s="392" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="Z7" s="392" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="AA7" s="392" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="AB7" s="392" t="n">
         <v>23</v>
       </c>
       <c r="AC7" s="392" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="AD7" s="392" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="AE7" s="392" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="AF7" s="392" t="n">
         <v>27</v>
@@ -24024,7 +24024,7 @@
     <row r="38" ht="12.75" customHeight="1" s="244">
       <c r="B38" s="411" t="inlineStr">
         <is>
-          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (25 devre): 201-1 (39.4 °C), 202-2 (41.1 °C), 202-3 (41.1 °C), 203-4 (39.9 °C), 204-5 (39.6 °C), 205-6 (39.3 °C), 205-7 (39.3 °C), 206-8 (32.4 °C) ...</t>
+          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (25 devre): 201-8 (39.4 °C), 202-3 (41.1 °C), 202-2 (41.1 °C), 203-4 (39.9 °C), 204-5 (39.6 °C), 205-6 (39.3 °C), 205-7 (39.3 °C), 206-9 (32.4 °C) ...</t>
         </is>
       </c>
       <c r="F38" s="243" t="inlineStr">

</xml_diff>

<commit_message>
STANDART: sihhi2 + yerden2 (kollektörlü, bloklar birebir) kullanıcı kaydıyla standart sistem; CLAUDE.md oturum talimatı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RwXcqZmf9VPBpDgb8LPkn3
</commit_message>
<xml_diff>
--- a/proje/denemeler/yerden2/NB_YERDEN_ISITMA.xlsx
+++ b/proje/denemeler/yerden2/NB_YERDEN_ISITMA.xlsx
@@ -12983,40 +12983,40 @@
       <c r="D7" s="389" t="n"/>
       <c r="E7" s="391" t="n"/>
       <c r="F7" s="392" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G7" s="392" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H7" s="392" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I7" s="392" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J7" s="392" t="n">
         <v>5</v>
       </c>
       <c r="K7" s="392" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L7" s="392" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="M7" s="392" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="N7" s="392" t="n">
         <v>9</v>
       </c>
       <c r="O7" s="392" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="P7" s="392" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q7" s="392" t="n">
         <v>11</v>
-      </c>
-      <c r="Q7" s="392" t="n">
-        <v>12</v>
       </c>
       <c r="R7" s="392" t="n">
         <v>13</v>
@@ -13031,37 +13031,37 @@
         <v>16</v>
       </c>
       <c r="V7" s="392" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="W7" s="392" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="X7" s="392" t="n">
         <v>19</v>
       </c>
       <c r="Y7" s="392" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="Z7" s="392" t="n">
         <v>21</v>
       </c>
       <c r="AA7" s="392" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="AB7" s="392" t="n">
+        <v>26</v>
+      </c>
+      <c r="AC7" s="392" t="n">
+        <v>27</v>
+      </c>
+      <c r="AD7" s="392" t="n">
         <v>23</v>
       </c>
-      <c r="AC7" s="392" t="n">
+      <c r="AE7" s="392" t="n">
+        <v>25</v>
+      </c>
+      <c r="AF7" s="392" t="n">
         <v>24</v>
-      </c>
-      <c r="AD7" s="392" t="n">
-        <v>25</v>
-      </c>
-      <c r="AE7" s="392" t="n">
-        <v>26</v>
-      </c>
-      <c r="AF7" s="392" t="n">
-        <v>27</v>
       </c>
     </row>
     <row r="8" ht="12" customHeight="1" s="244">
@@ -16081,7 +16081,7 @@
     <row r="38" ht="12.75" customHeight="1" s="244">
       <c r="B38" s="411" t="inlineStr">
         <is>
-          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): Z01-1 (39.9 °C), Z02-2 (40.8 °C), Z02-3 (40.8 °C), Z03-4 (39.8 °C), Z04-5 (39.7 °C), Z05-6 (39.2 °C), Z05-7 (39.2 °C), Z06-8 (29.8 °C) ...</t>
+          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): Z01-2 (39.9 °C), Z02-7 (40.8 °C), Z02-8 (40.8 °C), Z03-6 (39.8 °C), Z04-5 (39.7 °C), Z05-4 (39.2 °C), Z05-3 (39.2 °C), Z06-1 (29.8 °C) ...</t>
         </is>
       </c>
       <c r="H38" s="243" t="n"/>
@@ -16458,13 +16458,13 @@
       <c r="D7" s="389" t="n"/>
       <c r="E7" s="391" t="n"/>
       <c r="F7" s="392" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G7" s="392" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" s="392" t="n">
         <v>2</v>
-      </c>
-      <c r="H7" s="392" t="n">
-        <v>3</v>
       </c>
       <c r="I7" s="392" t="n">
         <v>4</v>
@@ -16479,61 +16479,61 @@
         <v>7</v>
       </c>
       <c r="M7" s="392" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N7" s="392" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="O7" s="392" t="n">
+        <v>18</v>
+      </c>
+      <c r="P7" s="392" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q7" s="392" t="n">
+        <v>11</v>
+      </c>
+      <c r="R7" s="392" t="n">
         <v>10</v>
       </c>
-      <c r="P7" s="392" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q7" s="392" t="n">
-        <v>12</v>
-      </c>
-      <c r="R7" s="392" t="n">
+      <c r="S7" s="392" t="n">
+        <v>15</v>
+      </c>
+      <c r="T7" s="392" t="n">
+        <v>16</v>
+      </c>
+      <c r="U7" s="392" t="n">
         <v>13</v>
-      </c>
-      <c r="S7" s="392" t="n">
-        <v>14</v>
-      </c>
-      <c r="T7" s="392" t="n">
-        <v>15</v>
-      </c>
-      <c r="U7" s="392" t="n">
-        <v>16</v>
       </c>
       <c r="V7" s="392" t="n">
         <v>17</v>
       </c>
       <c r="W7" s="392" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="X7" s="392" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Y7" s="392" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="Z7" s="392" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="AA7" s="392" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="AB7" s="392" t="n">
         <v>23</v>
       </c>
       <c r="AC7" s="392" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="AD7" s="392" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="AE7" s="392" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="AF7" s="392" t="n">
         <v>27</v>
@@ -20050,7 +20050,7 @@
     <row r="38" ht="12.75" customHeight="1" s="244">
       <c r="B38" s="411" t="inlineStr">
         <is>
-          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): 101-1 (39.9 °C), 102-2 (41.1 °C), 102-3 (41.1 °C), 103-4 (39.9 °C), 104-5 (39.6 °C), 105-6 (39.3 °C), 105-7 (39.3 °C), 106-8 (29.1 °C) ...</t>
+          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (27 devre): 101-8 (39.9 °C), 102-3 (41.1 °C), 102-2 (41.1 °C), 103-4 (39.9 °C), 104-5 (39.6 °C), 105-6 (39.3 °C), 105-7 (39.3 °C), 106-9 (29.1 °C) ...</t>
         </is>
       </c>
       <c r="F38" s="243" t="inlineStr">
@@ -20432,13 +20432,13 @@
       <c r="D7" s="389" t="n"/>
       <c r="E7" s="391" t="n"/>
       <c r="F7" s="392" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G7" s="392" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" s="392" t="n">
         <v>2</v>
-      </c>
-      <c r="H7" s="392" t="n">
-        <v>3</v>
       </c>
       <c r="I7" s="392" t="n">
         <v>4</v>
@@ -20453,61 +20453,61 @@
         <v>7</v>
       </c>
       <c r="M7" s="392" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N7" s="392" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="O7" s="392" t="n">
+        <v>18</v>
+      </c>
+      <c r="P7" s="392" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q7" s="392" t="n">
+        <v>11</v>
+      </c>
+      <c r="R7" s="392" t="n">
         <v>10</v>
       </c>
-      <c r="P7" s="392" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q7" s="392" t="n">
-        <v>12</v>
-      </c>
-      <c r="R7" s="392" t="n">
+      <c r="S7" s="392" t="n">
+        <v>16</v>
+      </c>
+      <c r="T7" s="392" t="n">
+        <v>17</v>
+      </c>
+      <c r="U7" s="392" t="n">
         <v>13</v>
       </c>
-      <c r="S7" s="392" t="n">
+      <c r="V7" s="392" t="n">
+        <v>15</v>
+      </c>
+      <c r="W7" s="392" t="n">
         <v>14</v>
       </c>
-      <c r="T7" s="392" t="n">
-        <v>15</v>
-      </c>
-      <c r="U7" s="392" t="n">
-        <v>16</v>
-      </c>
-      <c r="V7" s="392" t="n">
-        <v>17</v>
-      </c>
-      <c r="W7" s="392" t="n">
-        <v>18</v>
-      </c>
       <c r="X7" s="392" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Y7" s="392" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="Z7" s="392" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="AA7" s="392" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="AB7" s="392" t="n">
         <v>23</v>
       </c>
       <c r="AC7" s="392" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="AD7" s="392" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="AE7" s="392" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="AF7" s="392" t="n">
         <v>27</v>
@@ -24024,7 +24024,7 @@
     <row r="38" ht="12.75" customHeight="1" s="244">
       <c r="B38" s="411" t="inlineStr">
         <is>
-          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (25 devre): 201-1 (39.4 °C), 202-2 (41.1 °C), 202-3 (41.1 °C), 203-4 (39.9 °C), 204-5 (39.6 °C), 205-6 (39.3 °C), 205-7 (39.3 °C), 206-8 (32.4 °C) ...</t>
+          <t>UYARI: 35 W/m × L esasında döşeme yüzey sıcaklığı sınırı aşılıyor (25 devre): 201-8 (39.4 °C), 202-3 (41.1 °C), 202-2 (41.1 °C), 203-4 (39.9 °C), 204-5 (39.6 °C), 205-6 (39.3 °C), 205-7 (39.3 °C), 206-9 (32.4 °C) ...</t>
         </is>
       </c>
       <c r="F38" s="243" t="inlineStr">

</xml_diff>